<commit_message>
fix(ui): preserve fighter sessions and native dialog modes; refresh audited Excel
Publish exact source verified by 68 UI tests, 40 Fighter tests and 14 Chromium scenarios. Retain all game functions and initial 40-screen audit; document synthetic QA limitations. Include five-sheet workbook with refreshed evidence. Remove temporary review/transport scaffolding.
</commit_message>
<xml_diff>
--- a/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
+++ b/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R68a0d6fd0e094ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="R9e879afed5374d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="R50238ad93c314eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R6653a59432e3442d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="R74c14cbfb83e44a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R2c7b566fde3e40fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Re2b51408fa394e80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="Rc3d2b5f70a824259"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R73a011f5fdcc46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="Rca4d2bdb4fa34fc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -102,30 +102,16 @@
     </x:fill>
   </x:fills>
   <x:borders count="6">
+    <x:border/>
     <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:bottom>
-      <x:diagonal/>
     </x:border>
     <x:border>
-      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -134,27 +120,16 @@
       <x:right style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:right>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFFFFFFF"/>
       </x:left>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
     <x:border>
-      <x:left/>
-      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:top>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
@@ -312,7 +287,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -323,7 +298,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -334,7 +309,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +320,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -356,7 +331,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -367,7 +342,7 @@
         <x:color rgb="FFA31F2F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE7E7"/>
         </x:patternFill>
       </x:fill>
@@ -378,7 +353,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -389,7 +364,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -400,7 +375,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -411,7 +386,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -422,7 +397,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -433,7 +408,7 @@
         <x:color rgb="FFA31F2F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE7E7"/>
         </x:patternFill>
       </x:fill>
@@ -444,7 +419,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -455,7 +430,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -466,7 +441,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -477,7 +452,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -488,7 +463,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -499,7 +474,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -510,7 +485,7 @@
         <x:color rgb="FFA31F2F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE7E7"/>
         </x:patternFill>
       </x:fill>
@@ -521,7 +496,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -532,7 +507,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -543,7 +518,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -554,7 +529,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -565,7 +540,7 @@
         <x:color rgb="FF7B5100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CE"/>
         </x:patternFill>
       </x:fill>
@@ -576,7 +551,7 @@
         <x:color rgb="FFA31F2F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE7E7"/>
         </x:patternFill>
       </x:fill>
@@ -656,8 +631,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:H106"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:H114"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Réf."/>
     <x:tableColumn id="2" name="Nature de preuve"/>
@@ -914,7 +889,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>Audit 5f44cf34 · Base b8b2c326 · 2026-10-25</x:v>
+        <x:v>Audit initial 5f44cf34 · Base b8b2c326 · Reprise du 26 octobre 2026</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1041,7 +1016,7 @@
       </x:c>
       <x:c r="G10" s="35" t="n">
         <x:f>COUNTIFS('40 écrans'!$C$7:$C$46,A10,'40 écrans'!$F$7:$F$46,"Réussis")</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="H10" s="35" t="n">
         <x:f>COUNTIFS('40 écrans'!$C$7:$C$46,A10,'40 écrans'!$G$7:$G$46,"Observé sur branche")</x:f>
@@ -1107,7 +1082,7 @@
       </x:c>
       <x:c r="G12" s="41" t="n">
         <x:f>SUM(G9:G11)</x:f>
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H12" s="41" t="n">
         <x:f>SUM(H9:H11)</x:f>
@@ -1160,7 +1135,7 @@
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="46" t="str">
-        <x:v>Revue : perte de jauge PV Extinction détectée au prébuild ; jauge et PV max rétablis, tests noncombat réussis.</x:v>
+        <x:v>Reprise : stabilité du duel après pause/rendu parent ; vraie modalité native des panneaux ; preuves CI séparées de la recette visuelle.</x:v>
       </x:c>
       <x:c r="B16" s="2"/>
       <x:c r="C16" s="2"/>
@@ -1268,7 +1243,7 @@
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="46" t="str">
-        <x:v>Parcours CI adaptés aux nouveaux menus : 195 contrôles et attentes conservés ; résultat courant dans Vérifications.</x:v>
+        <x:v>Reprise vérifiée : 68 tests UI + 40 Fighter ; Chromium : 8 nouveaux parcours et 6 parcours existants réussis, avec données synthétiques.</x:v>
       </x:c>
       <x:c r="B25" s="2"/>
       <x:c r="C25" s="2"/>
@@ -1394,7 +1369,7 @@
       </x:c>
       <x:c r="B35" s="2"/>
       <x:c r="C35" s="47" t="str">
-        <x:v>Non renseigné — consulter le manifeste de validation</x:v>
+        <x:v>Source validée : run 40268408942 ; empreintes dans continuation-2026-10-26.json.</x:v>
       </x:c>
       <x:c r="D35" s="2"/>
       <x:c r="E35" s="2"/>
@@ -1437,7 +1412,7 @@
       </x:c>
       <x:c r="B38" s="2"/>
       <x:c r="C38" s="47" t="str">
-        <x:v>scripts/ui-immersion/build-workbook.sh — lit les ledgers et validation.json versionnés</x:v>
+        <x:v>Classeur actualisé par artifact_tool ; données de reprise : continuation-2026-10-26.json.</x:v>
       </x:c>
       <x:c r="D38" s="2"/>
       <x:c r="E38" s="2"/>
@@ -1457,7 +1432,7 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="7" t="str">
-        <x:v>Sources : audit-baseline.json + quatre ledgers d’implémentation + validation.json (si disponible).</x:v>
+        <x:v>Sources : audit-baseline.json, ledgers d’implémentation, validation.json et continuation-2026-10-26.json ; les preuves historiques restent conservées.</x:v>
       </x:c>
       <x:c r="B40" s="2"/>
       <x:c r="C40" s="2"/>
@@ -1469,7 +1444,7 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="7" t="str">
-        <x:v>Actualisation : 2026-10-25. Les liens de code suivent la branche, jusqu’à enregistrement du commit.</x:v>
+        <x:v>Actualisation : 2026-10-26. Recette réelle des 40 écrans non certifiée ; les scénarios CI utilisent des données de test.</x:v>
       </x:c>
       <x:c r="B41" s="2"/>
       <x:c r="C41" s="2"/>
@@ -3322,7 +3297,7 @@
       </x:c>
       <x:c r="G27" s="22" t="str">
         <x:f>IF(T27&lt;&gt;"Non réalisé",T27,IF(E27=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-02",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-02",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")=E27,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-02",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-02",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H27" s="22" t="str">
         <x:v>Le RPG partage une colonne centrée comprenant en-tête, barres, canvas et tableau d’actions. Le ciblage, l’attente ATB, les reliques et les panneaux propres aux rencontres existent déjà sous la scène.</x:v>
@@ -3399,10 +3374,10 @@
         <x:v>Passer à un champ de bataille plein viewport avec portraits, santé et ATB ancrés sur les bords, commandes contextuelles et cible clairement indiquée. Ouvrir inventaire et renseignements sans déplacer la scène hors de l’écran.</x:v>
       </x:c>
       <x:c r="S27" s="22" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>CI avec données synthétiques : consulter Vérifications et continuation-2026-10-26.json. Pas d’approbation visuelle complète.</x:v>
       </x:c>
       <x:c r="T27" s="22" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="363" customHeight="1">
@@ -3429,7 +3404,7 @@
       </x:c>
       <x:c r="G28" s="21" t="str">
         <x:f>IF(T28&lt;&gt;"Non réalisé",T28,IF(E28=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-03",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-03",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")=E28,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-03",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-03",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H28" s="21" t="str">
         <x:v>Le terrain tactique partage le cadre du GameCanvas et son panneau inférieur. Déplacement de caméra, zoom, annulation de visée, fin de tour, soutien et informations d’escorte sont déjà présents.</x:v>
@@ -3505,10 +3480,10 @@
         <x:v>Étendre le terrain au viewport, avec unité active et points d’action près des commandes, ordre des tours en bande compacte et objectif court. Montrer portées, trajectoires, couvertures et ressources dans le terrain ; garder le détail dans un inspecteur.</x:v>
       </x:c>
       <x:c r="S28" s="21" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>CI avec données synthétiques : consulter Vérifications et continuation-2026-10-26.json. Pas d’approbation visuelle complète.</x:v>
       </x:c>
       <x:c r="T28" s="21" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="376" customHeight="1">
@@ -3535,7 +3510,7 @@
       </x:c>
       <x:c r="G29" s="22" t="str">
         <x:f>IF(T29&lt;&gt;"Non réalisé",T29,IF(E29=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-04",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")=E29,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-01",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-04",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H29" s="22" t="str">
         <x:v>La mêlée utilise un canvas encadré et un panneau de contrôles externe. Remappage, manette et tactile existent déjà. L’annonce d’avant-match est rendue à la fois dans le DOM et au centre du canvas.</x:v>
@@ -3615,10 +3590,10 @@
         <x:v>Faire de l’arène le fond de jeu, avec informations des combattants, objectif et charges en HUD. Unifier l’annonce transitoire ; ranger aide et remappage dans Commandes et superposer les touches tactiles utiles.</x:v>
       </x:c>
       <x:c r="S29" s="22" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>CI avec données synthétiques : consulter Vérifications et continuation-2026-10-26.json. Pas d’approbation visuelle complète.</x:v>
       </x:c>
       <x:c r="T29" s="22" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="324" customHeight="1">
@@ -3641,18 +3616,18 @@
       </x:c>
       <x:c r="F30" s="21" t="str">
         <x:f>IF(E30=0,"Non réalisés",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$E$7:$E$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$E$7:$E$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$E$7:$E$45,"Bloqués")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$E$7:$E$45,"Bloqués")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$E$7:$E$45,"Partiels")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$E$7:$E$45,"Partiels")&gt;0,"Partiels",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$E$7:$E$45,"Réussis")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$E$7:$E$45,"Réussis")=E30,"Réussis",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$E$7:$E$45,"Réussis")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$E$7:$E$45,"Réussis")&gt;0,"Partiels",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$E$7:$E$45,"Déclarés")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$E$7:$E$45,"Déclarés")&gt;0,"Déclarés","Non réalisés"))))))</x:f>
-        <x:v>Partiels</x:v>
+        <x:v>Réussis</x:v>
       </x:c>
       <x:c r="G30" s="21" t="str">
         <x:f>IF(T30&lt;&gt;"Non réalisé",T30,IF(E30=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")=E30,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-05",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-08",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H30" s="21" t="str">
         <x:v>Fighter possède déjà son lobby, ses équipes, la difficulté ou le contrôle local adverse, puis une vue active avec canvas, panneau latéral et commandes. Remplaçants, supers, assistances et revanche sont disponibles.</x:v>
       </x:c>
       <x:c r="I30" s="21" t="str">
-        <x:v>COMBAT-05 — Préparation Fighter en composition versus avec le décor réel choisi et les portraits existants ; arène, musique, super terrain, adversaire, difficulté et lancement conservés.
-COMBAT-08 — Les recettes navigateur ouvrent le vrai bouton Arsenal avant les invocations, signatures de mêlée, reliques et soutiens tactiques. Elles referment le tiroir avant les actions du HUD et le rouvrent après une pause externe.</x:v>
+        <x:v>COMBAT-05 — Lobby versus et duel plein viewport ; état du moteur conservé malgré les rendus du parent, la pause et les options. Seule une revanche explicite reconstruit le duel avec les derniers réglages.
+COMBAT-08 — Scénarios navigateur synthétiques de régression maintenus et étendus.</x:v>
       </x:c>
       <x:c r="J30" s="21" t="str">
         <x:v>Conserver composition, changements de combattant, contrôle J2, difficulté, supers, assistances, résultat, revanche et retour au lobby. Le moteur sait déjà suivre la pause sans reconstruction.</x:v>
@@ -3661,10 +3636,7 @@
         <x:v>Un duel doit rester entièrement contrôlable sans scroll. J1 et J2 doivent garder leurs commandes séparées, les remplacements autorisés doivent rester identifiables et une revanche ne doit pas perdre la configuration.</x:v>
       </x:c>
       <x:c r="L30" s="21" t="str">
-        <x:v>Moteur, hitboxes, règles d’action et équilibre inchangés. Certification visuelle en attente de la preview commune.
-Aucune installation ni exécution locale du navigateur. Les recettes corrigées et la nouvelle vérification de libellé attendent la prochaine CI distante.
-Le portrait conserve toute l’arène horizontale et la réduit donc à l’écran. Le paysage est préférable pour les combats d’action ; caméra et géométrie du jeu restent inchangées.
-Les états initiaux sont synthétiques, avec les vrais composants et moteurs ; ils ne certifient ni un appareil physique ni un compte réel.</x:v>
+        <x:v>Les tests synthétiques contrôlent état, commandes et cycle de session, pas les illustrations ni le confort sur appareil physique. Le portrait conserve le ratio complet de l’arène.</x:v>
       </x:c>
       <x:c r="M30" s="21" t="str">
         <x:v>src/components/FighterMode.jsx
@@ -3713,10 +3685,10 @@
         <x:v>Utiliser un lobby visuel, puis une arène plein viewport avec barres, temps, remplaçants et charges intégrés au HUD. Déplacer les listes de commandes dans l’aide ; faire du résultat une transition de fin de duel.</x:v>
       </x:c>
       <x:c r="S30" s="21" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>CI avec données synthétiques : consulter Vérifications et continuation-2026-10-26.json. Pas d’approbation visuelle complète.</x:v>
       </x:c>
       <x:c r="T30" s="21" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="363" customHeight="1">
@@ -3743,19 +3715,13 @@
       </x:c>
       <x:c r="G31" s="22" t="str">
         <x:f>IF(T31&lt;&gt;"Non réalisé",T31,IF(E31=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-08",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-01",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-02",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-02",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")=E31,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-08",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-01",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-02",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-08",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-01",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-02",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-04",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H31" s="22" t="str">
         <x:v>Les sessions dédiées du hub ont déjà une pause avec reprise, abandon, Échap, focus et arrière-plan inactif. En revanche, le parcours campagne rend GameCanvas sans les propriétés qui raccordent cette pause.</x:v>
       </x:c>
       <x:c r="I31" s="22" t="str">
-        <x:v>HUB-08 — Barre dédiée de 56px superposée au monde et menu de pause existant conservé avec focus/inert.
-HUB-11 — La ref hubNavigationRef détenue par App conserve les choix d’interface entre les montages du Hub : destination, catégorie, mission de briefing, groupe/arc, sous-vues, filtres média/mode, recherches et statut du répertoire, recherche des groupes, héros sélectionné et pagination/filtres des cinq catalogues.
-HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.
-COMBAT-06 — GameCanvas et Fighter exposent onPauseRequest et composent pause externe et pause des dossiers ; le moteur reste monté et l’horloge est réinitialisée aux transitions.
-APP-01 — Préférences d’affichage persistantes séparées de la progression : texte, HUD, marge, contraste, mouvement.
-APP-02 — Audio, connexion, compte et sauvegardes regroupés dans le menu Système pour dégager les scènes.
-APP-04 — Pause commune aux missions de campagne, avec reprise, options, commandes et confirmation du repli.</x:v>
+        <x:v>Pause et paramètres conservent la session. Les tiroirs changent réellement de mode natif live/modal ; fermeture et démontage rétablissent le focus sans le voler lors des mises à jour.</x:v>
       </x:c>
       <x:c r="J31" s="22" t="str">
         <x:v>Préserver le gel de simulation, les confirmations d’abandon, le nettoyage des entrées et la restitution du focus. Une petite modale centrée reste adaptée à une pause courte.</x:v>
@@ -3781,29 +3747,10 @@
 Recette interactive du clavier/manette sur la preview à compléter.</x:v>
       </x:c>
       <x:c r="M31" s="22" t="str">
-        <x:v>src/components/HubScreen.jsx
-src/components/HubImmersion.css
-src/components/ImmersiveDrawer.jsx
-src/game/immersiveHubState.js
-scripts/immersiveHubState.test.mjs
-src/components/RaceMode.jsx
-src/components/useSceneViewport.js
-scripts/nonCombatTrial.test.mjs
-src/components/GameCanvas.jsx
-src/components/FighterMode.jsx
-src/components/CombatDrawer.jsx
-src/components/CombatResultDialog.jsx
-src/game/combatViewport.js
-scripts/combatViewport.test.mjs
-scripts/customBattle.test.mjs
-src/components/GameDisplaySettings.jsx
-src/game/displayPreferences.js
-src/components/game-system.css
-src/App.jsx
-src/components/GameSystemMenu.jsx
-src/components/GameSystemDialog.jsx
-src/game/gameDialogQueue.js
-src/components/CampaignPauseMenu.jsx</x:v>
+        <x:v>src/components/CombatDrawer.jsx
+src/game/combatDialogLifecycle.js
+scripts/combatDialogLifecycle.test.mjs
+scripts/browserImmersiveTransitions.py</x:v>
       </x:c>
       <x:c r="N31" s="22" t="str">
         <x:v>HUB-08, HUB-11, HUB-12, COMBAT-06, APP-01, APP-02, APP-04</x:v>
@@ -3826,10 +3773,10 @@
         <x:v>Réutiliser la pause existante dans les missions et unifier la navigation système. Donner accès aux options et à l’aide, avec retour à la session sans reconstruire le moteur ni changer son état.</x:v>
       </x:c>
       <x:c r="S31" s="22" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>CI avec données synthétiques : consulter Vérifications et continuation-2026-10-26.json. Pas d’approbation visuelle complète.</x:v>
       </x:c>
       <x:c r="T31" s="22" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="194" customHeight="1">
@@ -3856,7 +3803,7 @@
       </x:c>
       <x:c r="G32" s="21" t="str">
         <x:f>IF(T32&lt;&gt;"Non réalisé",T32,IF(E32=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-05",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"APP-06",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-05",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-06",Actions!$F$7:$F$45,"Observé sur branche")=E32,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-05",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"APP-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-11",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"COMBAT-06",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-05",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"APP-06",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H32" s="21" t="str">
         <x:v>Le résultat s’affiche dans le canvas, puis ouvre un débriefing riche. Hors session dédiée, le bouton de repli reste rendu alors que la victoire n’est transmise qu’après validation du résultat : risque de sortie comme abandon.</x:v>
@@ -3920,10 +3867,10 @@
         <x:v>Vérifier ce flux avant la refonte et sécuriser la sortie une fois le combat terminé. Présenter ensuite résultat, rang et gains, avec Butin, Performance, Conséquences et Journal en sous-vues.</x:v>
       </x:c>
       <x:c r="S32" s="21" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>CI avec données synthétiques : consulter Vérifications et continuation-2026-10-26.json. Pas d’approbation visuelle complète.</x:v>
       </x:c>
       <x:c r="T32" s="21" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="51" customHeight="1">
@@ -5001,7 +4948,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R583f164926794b50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d5586f08fed4098"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6737,29 +6684,24 @@
         <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G34" s="21" t="str">
-        <x:v>Préparation Fighter en composition versus avec le décor réel choisi et les portraits existants ; arène, musique, super terrain, adversaire, difficulté et lancement conservés.
-Duel couvrant le viewport au ratio logique 960 × 540 ; PV et chronomètre du moteur inchangés ; tags de banc compacts en surimpression.
-Supers terrain et assists dans un tiroir en direct ; commandes et affichage dans un tiroir suspendu ; barre d’arène accessible.
-Les deux joueurs gardent clavier et tactile. L’activation tactile est explicite et les appuis sont libérés à la perte de capture ou de focus.</x:v>
+        <x:v>Lobby versus et scène immersive conservés. Le moteur du duel est créé seulement au lancement ou à une revanche explicite ; les objets recréés par le parent ne réinitialisent plus PV, jauges, temps ou résultat. La prochaine rencontre lit les derniers réglages.</x:v>
       </x:c>
       <x:c r="H34" s="21" t="str">
         <x:v>src/components/FighterMode.jsx
-src/components/CombatDrawer.jsx
-src/components/combat-immersion.css</x:v>
+scripts/fixtures/fighterLifecycleHarness.jsx
+scripts/browserImmersiveTransitions.py</x:v>
       </x:c>
       <x:c r="I34" s="21" t="str">
-        <x:v>scripts/reauditFighterTagRoutes.test.mjs : 16/16 réussis sur les callbacks réels et le moteur Fighter ; deux côtés, trois emplacements, pause, onglet caché et hit-stop.
-Tests de remise à zéro d’horloge Fighter après pause et changement de visibilité réussis.
-Compilation JSX Fighter réussie.</x:v>
+        <x:v>68 tests UI ; 40 tests horloge/commandes ; 8/8 nouvelles recettes Chromium et 6/6 anciennes recettes Fighter. Source identique par SHA-256.</x:v>
       </x:c>
       <x:c r="J34" s="21" t="str">
-        <x:v>Moteur, hitboxes, règles d’action et équilibre inchangés. Certification visuelle en attente de la preview commune.</x:v>
+        <x:v>Moteur, hitboxes et équilibrage inchangés. Le navigateur utilise des combattants/états synthétiques : pas de certification artistique, de progression cloud ou de périphérique réel.</x:v>
       </x:c>
       <x:c r="K34" s="21" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
       </x:c>
       <x:c r="L34" s="27" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/FighterMode.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -6793,35 +6735,25 @@
         <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G35" s="22" t="str">
-        <x:v>GameCanvas et Fighter exposent onPauseRequest et composent pause externe et pause des dossiers ; le moteur reste monté et l’horloge est réinitialisée aux transitions.
-Les dialogues natifs isolent le focus pour les tiroirs suspendus et les bilans plein écran. Échap ne peut pas ouvrir une pause au-dessus d’un résultat.
-GameCanvas distingue verdict et acquittement : onSessionComplete annonce le verdict ; onBattleEnd est envoyé une seule fois après validation. Un repli tardif ne remplace pas une victoire ou une défaite.
-Fighter conserve onMatchComplete au verdict unique ; onSessionEnd attend Revanche ou Retour, pour garder l’enveloppe dédiée pendant le bilan.
-Le bilan conserve objectifs, récompenses, distinction Custom, pose, score, rang, durée, revanche et retour.</x:v>
+        <x:v>Pause, confirmations et résultat conservés. CombatDrawer referme le dialogue natif avant de passer de show() à showModal() ou inversement ; conserve l’élément d’ouverture et restaure le focus après fermeture/démontage.</x:v>
       </x:c>
       <x:c r="H35" s="22" t="str">
-        <x:v>src/components/GameCanvas.jsx
-src/components/FighterMode.jsx
-src/components/CombatDrawer.jsx
-src/components/CombatResultDialog.jsx
-src/game/combatViewport.js
-scripts/combatViewport.test.mjs
-scripts/customBattle.test.mjs</x:v>
+        <x:v>src/components/CombatDrawer.jsx
+src/game/combatDialogLifecycle.js
+scripts/combatDialogLifecycle.test.mjs
+scripts/fixtures/combatDrawerHarness.jsx</x:v>
       </x:c>
       <x:c r="I35" s="22" t="str">
-        <x:v>Les tests de garde du résultat rejettent un verdict prématuré, un résultat invalide, le repli tardif, la double validation et la finalisation après abandon.
-scripts/customBattle.test.mjs : 42/42 réussis ; entrée de pause et garde partagée vérifiées.
-scripts/fixedStepClock.test.mjs : 10/10 réussis.</x:v>
+        <x:v>9 nouveaux tests de dialogue inclus dans 68 tests UI. Quatre parcours Chromium passent : live↔modal, Échap, maintien de saisie et restitution du focus.</x:v>
       </x:c>
       <x:c r="J35" s="22" t="str">
-        <x:v>App reste responsable de l’attribution des récompenses de campagne ; sa garde indépendante est suivie dans le lot APP-05.
-Custom conserve l’enveloppe jusqu’à onBattleEnd ; intégration prise en charge dans le lot Hub.</x:v>
+        <x:v>Transitions natives testées indépendamment ; l’ensemble des combinaisons de menus et une campagne complète restent à parcourir en jeu.</x:v>
       </x:c>
       <x:c r="K35" s="22" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
       </x:c>
       <x:c r="L35" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/GameCanvas.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -6907,10 +6839,10 @@
         <x:v>Implémenté</x:v>
       </x:c>
       <x:c r="E37" s="23" t="str">
-        <x:v>Déclarés</x:v>
+        <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G37" s="22" t="str">
         <x:v>Les recettes navigateur ouvrent le vrai bouton Arsenal avant les invocations, signatures de mêlée, reliques et soutiens tactiques. Elles referment le tiroir avant les actions du HUD et le rouvrent après une pause externe.
@@ -6944,19 +6876,13 @@
 src/components/combat-immersion.css</x:v>
       </x:c>
       <x:c r="I37" s="22" t="str">
-        <x:v>Comparaison AST des assertions Python, attentes Playwright et attentes de simulation avec e2c03dd : les 195 obligations des neuf recettes existantes sont conservées. Une assertion de limites tactiles en portrait a été ajoutée.
-Python py_compile réussi pour les helpers et recettes de signature, RPG, Tactics et authentification.
-Les dix fixtures JSX ont été transformées par Vite transformWithOxc ; Oxlint et git diff --check réussis.
-Aucun nouveau clic forcé ni déclenchement JavaScript ajouté. Les régressions de double clic existantes restent inchangées ; la navigation ajoutée utilise les clics réguliers des locators Playwright.
-Captures CI synthétiques initiales examinées en desktop et portrait : le ratio conserve les acteurs visibles, avec des marges de décor sur écran haut.</x:v>
+        <x:v>Les trois workflows de la PR réussissent sur 92a8e247 (25/10/2026). Nouvelles transitions de cette reprise suivies séparément ; aucun ancien contrôle retiré.</x:v>
       </x:c>
       <x:c r="J37" s="22" t="str">
-        <x:v>Aucune installation ni exécution locale du navigateur. Les recettes corrigées et la nouvelle vérification de libellé attendent la prochaine CI distante.
-Le portrait conserve toute l’arène horizontale et la réduit donc à l’écran. Le paysage est préférable pour les combats d’action ; caméra et géométrie du jeu restent inchangées.
-Les états initiaux sont synthétiques, avec les vrais composants et moteurs ; ils ne certifient ni un appareil physique ni un compte réel.</x:v>
+        <x:v>CI navigateur avec vrais composants/moteurs et données synthétiques. Ne certifie pas la fidélité visuelle ni le tactile et les manettes réels.</x:v>
       </x:c>
       <x:c r="K37" s="22" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>Preuves CI et limites : docs/ui-immersion/continuation-2026-10-26.json ; recette réelle complète non effectuée.</x:v>
       </x:c>
       <x:c r="L37" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/scripts/browserCombatUi.py","Code de la branche"),"Code de la branche")</x:f>
@@ -7348,10 +7274,10 @@
         <x:v>Transversal</x:v>
       </x:c>
       <x:c r="D45" s="23" t="str">
-        <x:v>Partiel</x:v>
+        <x:v>Implémenté</x:v>
       </x:c>
       <x:c r="E45" s="23" t="str">
-        <x:v>Déclarés</x:v>
+        <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F45" s="23" t="str">
         <x:v>Non réalisé</x:v>
@@ -7366,14 +7292,13 @@
 docs/excel/Multiverse_Breach_UI_Immersion.xlsx</x:v>
       </x:c>
       <x:c r="I45" s="22" t="str">
-        <x:v>Compilation des sources réussie avec Vite 8.1.0 / Node 24.22.1.
-Suites de régression globales en cours.</x:v>
+        <x:v>CI de référence 92a8e247 : fiabilité, signatures et production réussies. Reprise : 68 tests UI, 40 Fighter, lint sans avertissement et compilation source réussis.</x:v>
       </x:c>
       <x:c r="J45" s="22" t="str">
-        <x:v>Prébuild complet des médias laissé à la CI du dépôt complet ; checkout local partiel.</x:v>
+        <x:v>La validation du commit final reste distincte des preuves de préparation. La recette complète avec médias, appareils et compte réel n’est pas déclarée faite.</x:v>
       </x:c>
       <x:c r="K45" s="22" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>Preuves CI et limites : docs/ui-immersion/continuation-2026-10-26.json ; recette réelle complète non effectuée.</x:v>
       </x:c>
       <x:c r="L45" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/package.json","Code de la branche"),"Code de la branche")</x:f>
@@ -7422,7 +7347,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5482ad1bd0ea4167"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R367e05ddb7704775"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8120,7 +8045,7 @@
       </x:c>
       <x:c r="F27" s="22" t="str">
         <x:f>'40 écrans'!G27</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G27" s="22" t="str">
         <x:v>Le joueur doit sélectionner une action et sa cible sans défilement. Les coordonnées doivent rester correctes après redimensionnement, et le mode d’attente doit garder exactement son comportement durant la sélection.</x:v>
@@ -8149,7 +8074,7 @@
       </x:c>
       <x:c r="F28" s="21" t="str">
         <x:f>'40 écrans'!G28</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G28" s="21" t="str">
         <x:v>Toutes les cases utiles doivent rester sélectionnables sans défilement de page. Panoramique et sélection doivent rester distincts, une annulation doit conserver les points d’action non dépensés et le HUD ne doit pas masquer la cible.</x:v>
@@ -8178,7 +8103,7 @@
       </x:c>
       <x:c r="F29" s="22" t="str">
         <x:f>'40 écrans'!G29</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G29" s="22" t="str">
         <x:v>Les entrées clavier, manette et tactile doivent rester équivalentes après déplacement des boutons. Une pause doit vider les commandes maintenues ; le HUD ne doit pas réduire la visibilité des bords de l’arène.</x:v>
@@ -8203,11 +8128,11 @@
       </x:c>
       <x:c r="E30" s="21" t="str">
         <x:f>'40 écrans'!F30</x:f>
-        <x:v>Partiels</x:v>
+        <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F30" s="21" t="str">
         <x:f>'40 écrans'!G30</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G30" s="21" t="str">
         <x:v>Un duel doit rester entièrement contrôlable sans scroll. J1 et J2 doivent garder leurs commandes séparées, les remplacements autorisés doivent rester identifiables et une revanche ne doit pas perdre la configuration.</x:v>
@@ -8236,7 +8161,7 @@
       </x:c>
       <x:c r="F31" s="22" t="str">
         <x:f>'40 écrans'!G31</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G31" s="22" t="str">
         <x:v>Vérifier séparément cité, course, Extinction, Fighter, custom et missions. Ouvrir un sous-menu puis reprendre doit conserver la scène, et un retour navigateur ou une perte de visibilité ne doit pas déclencher d’action involontaire.</x:v>
@@ -8265,7 +8190,7 @@
       </x:c>
       <x:c r="F32" s="21" t="str">
         <x:f>'40 écrans'!G32</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G32" s="21" t="str">
         <x:v>Fermer ou accélérer le résultat ne doit pas dupliquer les récompenses. Les gains doivent correspondre au profil, l’instabilité doit rester visible avant une nouvelle mission et le retour doit conduire au contexte attendu.</x:v>
@@ -8704,7 +8629,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ad29b27d6e6403c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd38e8f96e574234"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11069,28 +10994,28 @@
     </x:row>
     <x:row r="100" ht="51" customHeight="1">
       <x:c r="A100" s="21" t="str">
-        <x:v>CI-CURRENT</x:v>
+        <x:v>CI-92A8E247</x:v>
       </x:c>
       <x:c r="B100" s="21" t="str">
-        <x:v>CI distante</x:v>
+        <x:v>CI distante — référence</x:v>
       </x:c>
       <x:c r="C100" s="21" t="str">
-        <x:v>Non réalisé</x:v>
-      </x:c>
-      <x:c r="D100" s="21" t="str"/>
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D100" s="21" t="str">
+        <x:v>PR #9 avant reprise</x:v>
+      </x:c>
       <x:c r="E100" s="21" t="str">
-        <x:v>Workflows GitHub de la PR #9
-Nouvelle exécution attendue sur le commit des corrections et du classeur. Les contrôles de production ne sont ni supprimés ni contournés.</x:v>
+        <x:v>Trois workflows réussis : Reliability and source build ; Signature combat ; Full production build.</x:v>
       </x:c>
       <x:c r="F100" s="21" t="str">
-        <x:v>[]
-Résultat automatique : ne remplace pas la recette en appareil.</x:v>
+        <x:v>Commit 92a8e247a4b1bb296676aa17ea5b9c7e0bbd4dc6. Ne prouve pas à lui seul les modifications ultérieures.</x:v>
       </x:c>
       <x:c r="G100" s="21" t="str">
-        <x:v>https://github.com/darknigthmare/multiverse-breach/pull/9/checks</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40229637237</x:v>
       </x:c>
       <x:c r="H100" s="21" t="str">
-        <x:v>docs/ui-immersion/validation.json</x:v>
+        <x:v>GitHub Actions ; runs 40229637237, 40229637284, 40229637338</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="51" customHeight="1">
@@ -11235,6 +11160,212 @@
       <x:c r="G106" s="21" t="str"/>
       <x:c r="H106" s="21" t="str">
         <x:v>Plan de recette — audit initial et limites des ledgers</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="92" customHeight="1">
+      <x:c r="A107" t="str">
+        <x:v>REPRISE-UI</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>Tests automatiques</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>COMBAT-05, COMBAT-06, APP-08</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>npm run test:ui-immersion — 68/68, dont 9 nouveaux tests de cycle des dialogues.</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>Tests unitaires et contrats ; pas une recette jouée complète.</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>ui-tests.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="92" customHeight="1">
+      <x:c r="A108" t="str">
+        <x:v>REPRISE-FIGHTER</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>Tests automatiques</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>COMBAT-05</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>node --test scripts/fixedStepClock.test.mjs scripts/reauditFighterInputs.test.mjs — 40/40.</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>Horloge, commandes et cycle ; distinct des huit scénarios navigateur.</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>fighter-tests.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="92" customHeight="1">
+      <x:c r="A109" t="str">
+        <x:v>REPRISE-LINT</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>Analyse statique</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>6 modules/tests modifiés</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>oxlint --max-warnings 0 — zéro erreur et zéro avertissement.</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>N’analyse pas toutes les ressources du jeu.</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
+      </x:c>
+      <x:c r="H109" t="str">
+        <x:v>lint.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="92" customHeight="1">
+      <x:c r="A110" t="str">
+        <x:v>REPRISE-BUILD</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>Compilation source</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>Reprise UI</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>Vite build sur snapshot source : réussite.</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>Médias absents du snapshot ; avertissement de taille de chunk existant. Pas un build complet des médias.</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
+      </x:c>
+      <x:c r="H110" t="str">
+        <x:v>source-build.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="92" customHeight="1">
+      <x:c r="A111" t="str">
+        <x:v>REPRISE-BROWSER-1</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>Navigateur synthétique — historique</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>Partiel</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>COMBAT-05, COMBAT-06</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>4/8 scénarios réussis. Les quatre dialogues passent ; les quatre Fighter s’arrêtent au sélecteur exact des sliders.</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>Pas d’erreur JavaScript relevée. Sélecteurs corrigés et sliders manipulés au clavier dans la nouvelle recette.</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40267867939</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>transitions/results.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="92" customHeight="1">
+      <x:c r="A112" t="str">
+        <x:v>REPRISE-BROWSER-2</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>Navigateur synthétique</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>Fighter et CombatDrawer</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>8/8 scénarios réussis : Fighter + CombatDrawer, en 1280×900 FR, 390×844 EN, 844×390 FR et 2560×1080 EN. Pause, changements parent, réglages, bilan, revanche, modalité native et focus.</x:v>
+      </x:c>
+      <x:c r="F112" t="str">
+        <x:v>Régression de comportement sur vrais composants ; sans certification des médias, du cloud ou des périphériques physiques.</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
+      </x:c>
+      <x:c r="H112" t="str">
+        <x:v>scripts/browserImmersiveTransitions.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="92" customHeight="1">
+      <x:c r="A113" t="str">
+        <x:v>REPRISE-FIGHTER-EXISTANT</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>Navigateur synthétique</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>Fighter existant</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>6/6 scénarios Fighter existants : commandes J1/J2/IA, cycle du combat et deux erreurs injectées volontairement.</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>Exécution courante séparée des résultats unitaires ; aucune suppression de garde.</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40268408942</x:v>
+      </x:c>
+      <x:c r="H113" t="str">
+        <x:v>scripts/browserFighterLifecycle.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="92" customHeight="1">
+      <x:c r="A114" t="str">
+        <x:v>REPRISE-ENV</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>Environnement local</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>Bloqués</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>Navigation locale</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>Chromium local : ERR_BLOCKED_BY_ADMINISTRATOR ; recette déplacée vers le workflow GitHub.</x:v>
+      </x:c>
+      <x:c r="F114" t="str">
+        <x:v>Restriction d’environnement, pas un défaut du jeu. Aucune protection désactivée.</x:v>
+      </x:c>
+      <x:c r="G114"/>
+      <x:c r="H114" t="str">
+        <x:v>pr9-browser-transitions.log</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11260,7 +11391,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8169c4e1cf74f23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5373d678844432e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): preserve race sessions, held controls and portrait HUD; update audit workbook
Keep races stable across parent renders and garage upgrades, guard one-time results and recover from renderer faults. Add readable portrait telemetry without cropping the track. Verify 40 race-related tests, 68 existing UI tests and six Chromium scenarios with all seven race images. Publish the five-sheet Excel with 118 verification entries and remove temporary delivery scaffolding.
</commit_message>
<xml_diff>
--- a/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
+++ b/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R2c7b566fde3e40fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Re2b51408fa394e80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="Rc3d2b5f70a824259"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R73a011f5fdcc46b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="Rca4d2bdb4fa34fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R21a47f10c5224ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Rc2a442969f174d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="Rba7797ad8e4d467a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R63d5758042cf4ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="Rd510335fb9454930"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -135,7 +135,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="48">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -275,6 +275,13 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -631,8 +638,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:H114"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H124" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:H124"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Réf."/>
     <x:tableColumn id="2" name="Nature de preuve"/>
@@ -889,7 +896,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>Audit initial 5f44cf34 · Base b8b2c326 · Reprise du 26 octobre 2026</x:v>
+        <x:v>Audit initial 5f44cf34 · Base b8b2c326 · Suite Course du 26 octobre 2026</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1135,7 +1142,7 @@
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="46" t="str">
-        <x:v>Reprise : stabilité du duel après pause/rendu parent ; vraie modalité native des panneaux ; preuves CI séparées de la recette visuelle.</x:v>
+        <x:v>Suite Course : moteur conservé au garage, résultat unique, commandes maintenues et télémétrie portrait lisible.</x:v>
       </x:c>
       <x:c r="B16" s="2"/>
       <x:c r="C16" s="2"/>
@@ -1241,9 +1248,9 @@
       <x:c r="G24" s="2"/>
       <x:c r="H24" s="2"/>
     </x:row>
-    <x:row r="25" ht="22" customHeight="1">
+    <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="46" t="str">
-        <x:v>Reprise vérifiée : 68 tests UI + 40 Fighter ; Chromium : 8 nouveaux parcours et 6 parcours existants réussis, avec données synthétiques.</x:v>
+        <x:v>Course : 40 tests + 6 parcours Chromium hors ligne réussis. Les trois workflows de d45652f sont réussis. Détails et limites dans Vérifications.</x:v>
       </x:c>
       <x:c r="B25" s="2"/>
       <x:c r="C25" s="2"/>
@@ -1369,7 +1376,7 @@
       </x:c>
       <x:c r="B35" s="2"/>
       <x:c r="C35" s="47" t="str">
-        <x:v>Source validée : run 40268408942 ; empreintes dans continuation-2026-10-26.json.</x:v>
+        <x:v>Base d45652f ; sources, résultats et limites : race-continuation-2026-10-26.json.</x:v>
       </x:c>
       <x:c r="D35" s="2"/>
       <x:c r="E35" s="2"/>
@@ -1412,7 +1419,7 @@
       </x:c>
       <x:c r="B38" s="2"/>
       <x:c r="C38" s="47" t="str">
-        <x:v>Classeur actualisé par artifact_tool ; données de reprise : continuation-2026-10-26.json.</x:v>
+        <x:v>Actualisation artifact_tool ; historique du duel et suite Course conservés dans les deux comptes rendus de reprise.</x:v>
       </x:c>
       <x:c r="D38" s="2"/>
       <x:c r="E38" s="2"/>
@@ -1430,9 +1437,9 @@
       <x:c r="G39" s="2"/>
       <x:c r="H39" s="2"/>
     </x:row>
-    <x:row r="40">
+    <x:row r="40" ht="35" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>Sources : audit-baseline.json, ledgers d’implémentation, validation.json et continuation-2026-10-26.json ; les preuves historiques restent conservées.</x:v>
+        <x:v>Sources : audit initial, ledgers, validation.json, continuation-2026-10-26.json et race-continuation-2026-10-26.json.</x:v>
       </x:c>
       <x:c r="B40" s="2"/>
       <x:c r="C40" s="2"/>
@@ -1442,9 +1449,9 @@
       <x:c r="G40" s="2"/>
       <x:c r="H40" s="2"/>
     </x:row>
-    <x:row r="41">
+    <x:row r="41" ht="35" customHeight="1">
       <x:c r="A41" s="7" t="str">
-        <x:v>Actualisation : 2026-10-26. Recette réelle des 40 écrans non certifiée ; les scénarios CI utilisent des données de test.</x:v>
+        <x:v>26 octobre 2026 : Course testée sur composants réels avec états préparés ; médias et matériel physique non certifiés localement.</x:v>
       </x:c>
       <x:c r="B41" s="2"/>
       <x:c r="C41" s="2"/>
@@ -2984,13 +2991,14 @@
       </x:c>
       <x:c r="G23" s="22" t="str">
         <x:f>IF(T23&lt;&gt;"Non réalisé",T23,IF(E23=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Observé sur branche")=E23,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H23" s="22" t="str">
         <x:v>La préparation propose actuellement Mirelle Suture comme pilote, avec choix du châssis, du circuit et de l’aide d’autoaccélération. Ces décisions sont présentées comme un panneau de configuration plutôt qu’une grille de départ.</x:v>
       </x:c>
       <x:c r="I23" s="22" t="str">
-        <x:v>HUB-06 — Préparation conserve Mirelle, tous les châssis/circuits disponibles et l’accélération assistée. Garage, carrière, commandes et informations de circuit regroupés dans un terminal accessible avant et pendant la course.</x:v>
+        <x:v>HUB-06 — Préparation conserve Mirelle, tous les châssis/circuits disponibles et l’accélération assistée. Garage, carrière, commandes et informations de circuit regroupés dans un terminal accessible avant et pendant la course.
+Suite Course : stabilité du moteur/récompenses, pointeurs maintenus, reprise après erreur, télémétrie portrait visible.</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>Préserver tous les déblocages, choix de véhicule, aides et paramètres. Les achats et améliorations existants doivent rester accessibles dans le garage, sans être supprimés pour simplifier la présentation.</x:v>
@@ -2999,9 +3007,7 @@
         <x:v>Lancement et retour doivent conserver le pilote, le châssis, le circuit et les aides. Le joueur doit comprendre ce qui est disponible, équipé ou verrouillé sans devoir essayer chaque sélection.</x:v>
       </x:c>
       <x:c r="L23" s="22" t="str">
-        <x:v>Le ratio physique du moteur de course reste 16:9 : bandes de fond possibles sur portrait ou ultralarge, afin de conserver cadrage et collisions.
-Le compteur de temps/objectif accessible est conservé dans le DOM ; les jauges graphiques existantes restent dessinées par le moteur.
-Une course complète et un achat de garage via la preview restent à vérifier.</x:v>
+        <x:v>Observation partielle sur fixture Chromium, sans visite complète de la preview ni certification des médias. Le ratio/cadrage du moteur est conservé. Les essais manette, multitouch physique, cloud et tous circuits restent ouverts.</x:v>
       </x:c>
       <x:c r="M23" s="22" t="str">
         <x:v>src/components/RaceMode.jsx
@@ -3029,10 +3035,10 @@
         <x:v>Utiliser un garage ou une grille plein écran avec le kart sélectionné, Mirelle et un aperçu du circuit. Ranger les réglages complémentaires dans leurs rubriques et garder un résumé de course avant lancement.</x:v>
       </x:c>
       <x:c r="S23" s="22" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>26/10 : parcours Chromium isolés sur Course ; contrôle du garage, conduite, résultat et erreurs. Vrais composants, sans médias locaux ni compte réel.</x:v>
       </x:c>
       <x:c r="T23" s="22" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="168" customHeight="1">
@@ -3059,14 +3065,15 @@
       </x:c>
       <x:c r="G24" s="21" t="str">
         <x:f>IF(T24&lt;&gt;"Non réalisé",T24,IF(E24=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")=E24,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H24" s="21" t="str">
         <x:v>La course utilise un canvas avec panneau latéral contenant statistiques, carrière, objectif, objet, garage, circuit et aide. Un texte de développement est encore placé dans l’en-tête de la vue active.</x:v>
       </x:c>
       <x:c r="I24" s="21" t="str">
         <x:v>HUB-06 — Préparation conserve Mirelle, tous les châssis/circuits disponibles et l’accélération assistée. Garage, carrière, commandes et informations de circuit regroupés dans un terminal accessible avant et pendant la course.
-HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.</x:v>
+HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.
+Suite Course : stabilité du moteur/récompenses, pointeurs maintenus, reprise après erreur, télémétrie portrait visible.</x:v>
       </x:c>
       <x:c r="J24" s="21" t="str">
         <x:v>Conserver objet actif, aides, statistiques, carrière et garage. Réécrire les messages de développement en indications utiles au joueur, tout en laissant les détails techniques accessibles dans les outils.</x:v>
@@ -3075,12 +3082,7 @@
         <x:v>Les virages et concurrents doivent rester visibles derrière le HUD. Aucun achat ne doit détourner une commande de conduite, et l’ouverture d’une pause ne doit ni avancer la course ni réinitialiser le véhicule.</x:v>
       </x:c>
       <x:c r="L24" s="21" t="str">
-        <x:v>Le ratio physique du moteur de course reste 16:9 : bandes de fond possibles sur portrait ou ultralarge, afin de conserver cadrage et collisions.
-Le compteur de temps/objectif accessible est conservé dans le DOM ; les jauges graphiques existantes restent dessinées par le moteur.
-Une course complète et un achat de garage via la preview restent à vérifier.
-La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
-Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.</x:v>
+        <x:v>Observation partielle sur fixture Chromium, sans visite complète de la preview ni certification des médias. Le ratio/cadrage du moteur est conservé. Les essais manette, multitouch physique, cloud et tous circuits restent ouverts.</x:v>
       </x:c>
       <x:c r="M24" s="21" t="str">
         <x:v>src/components/RaceMode.jsx
@@ -3113,10 +3115,10 @@
         <x:v>Donner toute la surface à la piste, avec classement, tour, temps, vitesse et objet dans un HUD compact. Déplacer carrière, achats, améliorations et descriptions vers la préparation ou la pause ; garder les commandes tactiles adaptées.</x:v>
       </x:c>
       <x:c r="S24" s="21" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>26/10 : parcours Chromium isolés sur Course ; contrôle du garage, conduite, résultat et erreurs. Vrais composants, sans médias locaux ni compte réel.</x:v>
       </x:c>
       <x:c r="T24" s="21" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="168" customHeight="1">
@@ -3143,14 +3145,15 @@
       </x:c>
       <x:c r="G25" s="22" t="str">
         <x:f>IF(T25&lt;&gt;"Non réalisé",T25,IF(E25=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")=E25,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-06",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H25" s="22" t="str">
         <x:v>La course affiche déjà un bandeau de fin avec rang, temps, objectif et récompenses. Ce résultat reste intégré à la composition actuelle du canvas et de son environnement de panneaux.</x:v>
       </x:c>
       <x:c r="I25" s="22" t="str">
         <x:v>HUB-06 — Préparation conserve Mirelle, tous les châssis/circuits disponibles et l’accélération assistée. Garage, carrière, commandes et informations de circuit regroupés dans un terminal accessible avant et pendant la course.
-HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.</x:v>
+HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.
+Suite Course : stabilité du moteur/récompenses, pointeurs maintenus, reprise après erreur, télémétrie portrait visible.</x:v>
       </x:c>
       <x:c r="J25" s="22" t="str">
         <x:v>Conserver toutes les statistiques et récompenses de carrière existantes ainsi que la progression enregistrée. Le résultat ne doit pas devenir une seconde occasion d’appliquer les mêmes gains.</x:v>
@@ -3159,12 +3162,7 @@
         <x:v>Les valeurs annoncées doivent correspondre à la carrière après fermeture. Rejouer doit conserver la configuration voulue, changer de circuit doit retrouver le garage, et quitter doit rendre le contrôle au bon menu.</x:v>
       </x:c>
       <x:c r="L25" s="22" t="str">
-        <x:v>Le ratio physique du moteur de course reste 16:9 : bandes de fond possibles sur portrait ou ultralarge, afin de conserver cadrage et collisions.
-Le compteur de temps/objectif accessible est conservé dans le DOM ; les jauges graphiques existantes restent dessinées par le moteur.
-Une course complète et un achat de garage via la preview restent à vérifier.
-La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
-Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.</x:v>
+        <x:v>Observation partielle sur fixture Chromium, sans visite complète de la preview ni certification des médias. Le ratio/cadrage du moteur est conservé. Les essais manette, multitouch physique, cloud et tous circuits restent ouverts.</x:v>
       </x:c>
       <x:c r="M25" s="22" t="str">
         <x:v>src/components/RaceMode.jsx
@@ -3196,10 +3194,10 @@
         <x:v>Présenter un podium ou un bilan sur la scène, avec place, temps et gains immédiatement lisibles, puis un détail de carrière ouvrable. Mettre Rejouer, Changer de circuit et Quitter dans une zone d’action stable.</x:v>
       </x:c>
       <x:c r="S25" s="22" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>26/10 : parcours Chromium isolés sur Course ; contrôle du garage, conduite, résultat et erreurs. Vrais composants, sans médias locaux ni compte réel.</x:v>
       </x:c>
       <x:c r="T25" s="22" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="51" customHeight="1">
@@ -4948,7 +4946,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d5586f08fed4098"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R329e0c628dc54133"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6035,43 +6033,48 @@
         <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F23" s="23" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G23" s="22" t="str">
         <x:v>Préparation conserve Mirelle, tous les châssis/circuits disponibles et l’accélération assistée. Garage, carrière, commandes et informations de circuit regroupés dans un terminal accessible avant et pendant la course.
 Le terminal de course suspend réellement l’horloge et vide les touches maintenues. Une amélioration met à jour le moteur existant au lieu de redémarrer une course.
 Scène de course sur tout le viewport, cadre caméra 960×540 conservé sans déformation, HUD et actions contextuelles superposés.
-Bilan conservé en scène jusqu’à Rejouer ou Changer de circuit ; les contrôles de la course derrière le bilan deviennent inertes.</x:v>
+Bilan conservé en scène jusqu’à Rejouer ou Changer de circuit ; les contrôles de la course derrière le bilan deviennent inertes.
+Suite du 26/10 : correction du redémarrage involontaire lors d’un rendu parent ou d’un achat garage. Revanche explicite avec nouvelle session, sans récompenser les anciens callbacks. Maintien des touches par pointeur ; relâchement hors bouton et activation clavier séparés. Écran de récupération après erreur de rendu. HUD portrait visible et agrandissable ; cache remise à zéro à la revanche.</x:v>
       </x:c>
       <x:c r="H23" s="22" t="str">
         <x:v>src/components/RaceMode.jsx
 src/components/HubScreen.jsx
 src/components/HubImmersion.css
 src/components/ImmersiveDrawer.jsx
-scripts/fixedStepClock.test.mjs</x:v>
+scripts/fixedStepClock.test.mjs
+src/game/raceSessionControls.js
+scripts/raceSessionControls.test.mjs
+scripts/browserRaceImmersion.py
+scripts/fixtures/raceLifecycleHarness.jsx
+.github/workflows/race-ui.yml</x:v>
       </x:c>
       <x:c r="I23" s="22" t="str">
         <x:v>Tests fighterRaceGameplayAudit et kartCareerSave réussis.
 fixedStepClock enrichi : ouverture/fermeture garage ne reconstruit pas le moteur et ne rattrape pas le temps suspendu.
 Oxlint sur les six sources du lot : succès, aucun avertissement.
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
-git diff --check : succès.</x:v>
+git diff --check : succès.
+Suite Course : 40/40 tests unitaires, 6/6 parcours Chromium hors ligne ; aucun avertissement de lint sur les six modules/tests modifiés. Échec avant correction reproduit : moteur recréé par le parent et par l’achat ; corrigé avec assertions sur l’identité du moteur, le temps et le tour.</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
-        <x:v>Le ratio physique du moteur de course reste 16:9 : bandes de fond possibles sur portrait ou ultralarge, afin de conserver cadrage et collisions.
-Le compteur de temps/objectif accessible est conservé dans le DOM ; les jauges graphiques existantes restent dessinées par le moteur.
-Une course complète et un achat de garage via la preview restent à vérifier.</x:v>
+        <x:v>Ratio 16:9 conservé : bandes de fond possibles sans recadrage. Six parcours isolés, carrière préparée et deux erreurs injectées ; ce n’est pas une campagne complète. La télémétrie portrait est lisible dans le DOM, mais des libellés du moteur restent en français. Absence locale des médias ; contrôle des sept images requis par le nouveau workflow. Manette, multitouch réel et cloud restent non testés.</x:v>
       </x:c>
       <x:c r="K23" s="22" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>Capture et résultats Chromium hors ligne : race-ui-qa/browser-final ; 390×844, 844×390, 1280×900, 2560×1080. Composants réels, données et résultat préparés.</x:v>
       </x:c>
       <x:c r="L23" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/RaceMode.jsx","Code de la branche"),"Code de la branche")</x:f>
         <x:v>Code de la branche</x:v>
       </x:c>
       <x:c r="M23" s="26" t="str">
-        <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/hub-implementation.json","HUB-06"),"HUB-06")</x:f>
-        <x:v>HUB-06</x:v>
+        <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json","Suite Course et preuves"),"Suite Course et preuves")</x:f>
+        <x:v>Suite Course et preuves</x:v>
       </x:c>
       <x:c r="N23" s="22" t="str">
         <x:v>S17;S18;S19;</x:v>
@@ -7347,7 +7350,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R367e05ddb7704775"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f20f6069fb408d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7929,7 +7932,7 @@
       </x:c>
       <x:c r="F23" s="22" t="str">
         <x:f>'40 écrans'!G23</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G23" s="22" t="str">
         <x:v>Lancement et retour doivent conserver le pilote, le châssis, le circuit et les aides. Le joueur doit comprendre ce qui est disponible, équipé ou verrouillé sans devoir essayer chaque sélection.</x:v>
@@ -7958,7 +7961,7 @@
       </x:c>
       <x:c r="F24" s="21" t="str">
         <x:f>'40 écrans'!G24</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G24" s="21" t="str">
         <x:v>Les virages et concurrents doivent rester visibles derrière le HUD. Aucun achat ne doit détourner une commande de conduite, et l’ouverture d’une pause ne doit ni avancer la course ni réinitialiser le véhicule.</x:v>
@@ -7987,7 +7990,7 @@
       </x:c>
       <x:c r="F25" s="22" t="str">
         <x:f>'40 écrans'!G25</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G25" s="22" t="str">
         <x:v>Les valeurs annoncées doivent correspondre à la carrière après fermeture. Rejouer doit conserver la configuration voulue, changer de circuit doit retrouver le garage, et quitter doit rendre le contrôle au bon menu.</x:v>
@@ -8629,7 +8632,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd38e8f96e574234"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07df8ff7298241bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11368,6 +11371,266 @@
         <x:v>pr9-browser-transitions.log</x:v>
       </x:c>
     </x:row>
+    <x:row r="115" ht="104" customHeight="1">
+      <x:c r="A115" s="50" t="str">
+        <x:v>COURSE-BASE-FIABILITE</x:v>
+      </x:c>
+      <x:c r="B115" s="50" t="str">
+        <x:v>CI historique sur d45652f</x:v>
+      </x:c>
+      <x:c r="C115" s="50" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D115" s="50" t="str">
+        <x:v>Fiabilité / UI antérieure</x:v>
+      </x:c>
+      <x:c r="E115" s="50" t="str">
+        <x:v>Workflow Reliability and source build terminé avec succès.</x:v>
+      </x:c>
+      <x:c r="F115" s="50" t="str">
+        <x:v>Contrôle du commit précédent, pas preuve du nouveau patch Course.</x:v>
+      </x:c>
+      <x:c r="G115" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40269423554</x:v>
+      </x:c>
+      <x:c r="H115" s="50" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="104" customHeight="1">
+      <x:c r="A116" s="50" t="str">
+        <x:v>COURSE-BASE-SIGNATURES</x:v>
+      </x:c>
+      <x:c r="B116" s="50" t="str">
+        <x:v>CI historique sur d45652f</x:v>
+      </x:c>
+      <x:c r="C116" s="50" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D116" s="50" t="str">
+        <x:v>Signatures de combat</x:v>
+      </x:c>
+      <x:c r="E116" s="50" t="str">
+        <x:v>Workflow Signature combat terminé avec succès.</x:v>
+      </x:c>
+      <x:c r="F116" s="50" t="str">
+        <x:v>Contrôle du commit précédent, pas preuve du nouveau patch Course.</x:v>
+      </x:c>
+      <x:c r="G116" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40269423464</x:v>
+      </x:c>
+      <x:c r="H116" s="50" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="104" customHeight="1">
+      <x:c r="A117" s="50" t="str">
+        <x:v>COURSE-BASE-BUILD</x:v>
+      </x:c>
+      <x:c r="B117" s="50" t="str">
+        <x:v>CI historique sur d45652f</x:v>
+      </x:c>
+      <x:c r="C117" s="50" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D117" s="50" t="str">
+        <x:v>Build complet</x:v>
+      </x:c>
+      <x:c r="E117" s="50" t="str">
+        <x:v>Workflow Full production build terminé avec succès.</x:v>
+      </x:c>
+      <x:c r="F117" s="50" t="str">
+        <x:v>N’est pas une promotion en production ; ne valide pas artistiquement les 40 écrans.</x:v>
+      </x:c>
+      <x:c r="G117" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40269423586</x:v>
+      </x:c>
+      <x:c r="H117" s="50" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="104" customHeight="1">
+      <x:c r="A118" s="50" t="str">
+        <x:v>COURSE-REPRO</x:v>
+      </x:c>
+      <x:c r="B118" s="50" t="str">
+        <x:v>Régression reproduite puis corrigée</x:v>
+      </x:c>
+      <x:c r="C118" s="50" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D118" s="50" t="str">
+        <x:v>HUB-06 / écrans 17–19</x:v>
+      </x:c>
+      <x:c r="E118" s="50" t="str">
+        <x:v>Avant : moteur 0 → 1 après rendu parent → 2 après achat. Après : même moteur, temps/tour/position conservés.</x:v>
+      </x:c>
+      <x:c r="F118" s="50" t="str">
+        <x:v>Fixture réelle RaceMode/EngineRace avec carrière préparée ; 300 pièces initiales.</x:v>
+      </x:c>
+      <x:c r="G118" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H118" s="50" t="str">
+        <x:v>before/reproduction.json ; after-reproduction.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="104" customHeight="1">
+      <x:c r="A119" s="50" t="str">
+        <x:v>COURSE-UNIT</x:v>
+      </x:c>
+      <x:c r="B119" s="50" t="str">
+        <x:v>Tests automatiques</x:v>
+      </x:c>
+      <x:c r="C119" s="50" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D119" s="50" t="str">
+        <x:v>HUB-06 / entrées, carrière, horloge</x:v>
+      </x:c>
+      <x:c r="E119" s="50" t="str">
+        <x:v>40/40 tests, dont 9 nouveaux : réception unique, session périmée, indépendance des pointeurs et du clavier.</x:v>
+      </x:c>
+      <x:c r="F119" s="50" t="str">
+        <x:v>Cas de simulation ; ne remplace pas un périphérique physique.</x:v>
+      </x:c>
+      <x:c r="G119" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H119" s="50" t="str">
+        <x:v>unit-final.log ; scripts/raceSessionControls.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="104" customHeight="1">
+      <x:c r="A120" s="50" t="str">
+        <x:v>COURSE-BROWSER</x:v>
+      </x:c>
+      <x:c r="B120" s="50" t="str">
+        <x:v>Navigateur isolé hors ligne</x:v>
+      </x:c>
+      <x:c r="C120" s="50" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D120" s="50" t="str">
+        <x:v>Course / quatre formats / FR–EN</x:v>
+      </x:c>
+      <x:c r="E120" s="50" t="str">
+        <x:v>6/6 : garage, pause, rendu parent, pointeur hors bouton, activation clavier, bilan unique, revanche, démontage et deux erreurs de rendu injectées.</x:v>
+      </x:c>
+      <x:c r="F120" s="50" t="str">
+        <x:v>IIFE/CSS sur about:blank, stockage en mémoire, données préparées ; aucun média validé localement.</x:v>
+      </x:c>
+      <x:c r="G120" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H120" s="50" t="str">
+        <x:v>scripts/browserRaceImmersion.py ; browser-final/results.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="104" customHeight="1">
+      <x:c r="A121" s="50" t="str">
+        <x:v>COURSE-LINT</x:v>
+      </x:c>
+      <x:c r="B121" s="50" t="str">
+        <x:v>Analyse statique</x:v>
+      </x:c>
+      <x:c r="C121" s="50" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D121" s="50" t="str">
+        <x:v>Six modules/tests modifiés</x:v>
+      </x:c>
+      <x:c r="E121" s="50" t="str">
+        <x:v>Oxlint --max-warnings 0 : zéro erreur et zéro avertissement.</x:v>
+      </x:c>
+      <x:c r="F121" s="50" t="str">
+        <x:v>Pas une analyse de tous les médias ni de toute la base.</x:v>
+      </x:c>
+      <x:c r="G121" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H121" s="50" t="str">
+        <x:v>lint-final.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="104" customHeight="1">
+      <x:c r="A122" s="50" t="str">
+        <x:v>COURSE-HUD</x:v>
+      </x:c>
+      <x:c r="B122" s="50" t="str">
+        <x:v>Inspection de captures isolées</x:v>
+      </x:c>
+      <x:c r="C122" s="50" t="str">
+        <x:v>Partiel</x:v>
+      </x:c>
+      <x:c r="D122" s="50" t="str">
+        <x:v>Portrait et paysage court</x:v>
+      </x:c>
+      <x:c r="E122" s="50" t="str">
+        <x:v>Télémétrie portrait visible à 390×844, échelle HUD 1,2 ; résultat et actions accessibles à 844×390.</x:v>
+      </x:c>
+      <x:c r="F122" s="50" t="str">
+        <x:v>Rendu sans images, pas une recette artistique. Les libellés moteur non localisés restent à reprendre.</x:v>
+      </x:c>
+      <x:c r="G122" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H122" s="50" t="str">
+        <x:v>browser-final/*-race.png ; *-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="104" customHeight="1">
+      <x:c r="A123" s="50" t="str">
+        <x:v>COURSE-CI</x:v>
+      </x:c>
+      <x:c r="B123" s="50" t="str">
+        <x:v>Automatisation ajoutée</x:v>
+      </x:c>
+      <x:c r="C123" s="50" t="str">
+        <x:v>Déclarés</x:v>
+      </x:c>
+      <x:c r="D123" s="50" t="str">
+        <x:v>Nouveau workflow Race immersive UI</x:v>
+      </x:c>
+      <x:c r="E123" s="50" t="str">
+        <x:v>Exécute les 40 tests et 6 parcours avec --require-art ; exige le chargement des sept images du moteur.</x:v>
+      </x:c>
+      <x:c r="F123" s="50" t="str">
+        <x:v>État à la préparation du classeur : non exécuté sur le commit final. Résultat courant à consulter dans Checks.</x:v>
+      </x:c>
+      <x:c r="G123" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/pull/9/checks</x:v>
+      </x:c>
+      <x:c r="H123" s="50" t="str">
+        <x:v>.github/workflows/race-ui.yml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="104" customHeight="1">
+      <x:c r="A124" s="50" t="str">
+        <x:v>COURSE-LIMITES</x:v>
+      </x:c>
+      <x:c r="B124" s="50" t="str">
+        <x:v>Recette restant à réaliser</x:v>
+      </x:c>
+      <x:c r="C124" s="50" t="str">
+        <x:v>Non réalisés</x:v>
+      </x:c>
+      <x:c r="D124" s="50" t="str">
+        <x:v>Matériel / progression / 40 écrans</x:v>
+      </x:c>
+      <x:c r="E124" s="50" t="str">
+        <x:v>Manette physique, multitouch réel, vrai compte cloud, parcours de chaque circuit et recette artistique globale.</x:v>
+      </x:c>
+      <x:c r="F124" s="50" t="str">
+        <x:v>Ne sont pas marqués terminés par les suites automatisées.</x:v>
+      </x:c>
+      <x:c r="G124" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H124" s="50" t="str">
+        <x:v>Périmètre de livraison</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C7:C106">
     <x:cfRule type="cellIs" dxfId="19" priority="1" operator="equal">
@@ -11389,9 +11652,14 @@
       <x:formula>"Échec"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C115:C124">
+      <x:formula1>"Réussis,Partiel,Échec,Bloqués,Déclarés,Non réalisés"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5373d678844432e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c8a79faed344ad3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(ui): publish City and Extinction Excel with 132 checks and verified evidence
Keep all 40 screen records and prior history; separate tested behaviour from remaining visual and physical-device QA. Publish exact verified workbook and source receipts. Remove temporary workbook transport files and workflow.
</commit_message>
<xml_diff>
--- a/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
+++ b/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R21a47f10c5224ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Rc2a442969f174d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="Rba7797ad8e4d467a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R63d5758042cf4ee0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="Rd510335fb9454930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Rfdf25aa27a084d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Rd9968c246a79403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="R109e97c4eb404e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="Ra05bd74ebf314381"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="R326bc93759ed4779"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -638,8 +638,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H124" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:H124"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H138" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:H138"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Réf."/>
     <x:tableColumn id="2" name="Nature de preuve"/>
@@ -896,7 +896,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>Audit initial 5f44cf34 · Base b8b2c326 · Suite Course du 26 octobre 2026</x:v>
+        <x:v>Suivi continu de l’audit des 40 écrans — suite Cité et Extinction du 26 octobre 2026.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1142,7 +1142,7 @@
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="46" t="str">
-        <x:v>Suite Course : moteur conservé au garage, résultat unique, commandes maintenues et télémétrie portrait lisible.</x:v>
+        <x:v>Cité : déplacements, terminal, habitants et reprise. Extinction : entrées, visée, Directive, HUD, bilan modal et erreurs. Fonctions et contenus conservés.</x:v>
       </x:c>
       <x:c r="B16" s="2"/>
       <x:c r="C16" s="2"/>
@@ -1250,7 +1250,7 @@
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="46" t="str">
-        <x:v>Course : 40 tests + 6 parcours Chromium hors ligne réussis. Les trois workflows de d45652f sont réussis. Détails et limites dans Vérifications.</x:v>
+        <x:v>Suite Cité/Extinction : 64 tests ciblés, 68 tests UI et 10 parcours Chromium réussis ; suites unitaires se recoupant. Quatre formats, FR/EN, vrais médias, fins préparées.</x:v>
       </x:c>
       <x:c r="B25" s="2"/>
       <x:c r="C25" s="2"/>
@@ -1376,7 +1376,7 @@
       </x:c>
       <x:c r="B35" s="2"/>
       <x:c r="C35" s="47" t="str">
-        <x:v>Base d45652f ; sources, résultats et limites : race-continuation-2026-10-26.json.</x:v>
+        <x:v>Base c10f75b / snapshot 80468d2 ; nouvelle preuve : city-extinction-continuation-2026-10-26.json.</x:v>
       </x:c>
       <x:c r="D35" s="2"/>
       <x:c r="E35" s="2"/>
@@ -1419,7 +1419,7 @@
       </x:c>
       <x:c r="B38" s="2"/>
       <x:c r="C38" s="47" t="str">
-        <x:v>Actualisation artifact_tool ; historique du duel et suite Course conservés dans les deux comptes rendus de reprise.</x:v>
+        <x:v>Actualisation artifact_tool ; historique Fighter, Course et Cité/Extinction conservé. Les seuls ledgers initiaux ne reproduisent pas les annotations des reprises.</x:v>
       </x:c>
       <x:c r="D38" s="2"/>
       <x:c r="E38" s="2"/>
@@ -1439,7 +1439,7 @@
     </x:row>
     <x:row r="40" ht="35" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>Sources : audit initial, ledgers, validation.json, continuation-2026-10-26.json et race-continuation-2026-10-26.json.</x:v>
+        <x:v>Sources : audit initial, ledgers, validation.json et comptes rendus de reprise Fighter, Course, Cité/Extinction.</x:v>
       </x:c>
       <x:c r="B40" s="2"/>
       <x:c r="C40" s="2"/>
@@ -1451,7 +1451,7 @@
     </x:row>
     <x:row r="41" ht="35" customHeight="1">
       <x:c r="A41" s="7" t="str">
-        <x:v>26 octobre 2026 : Course testée sur composants réels avec états préparés ; médias et matériel physique non certifiés localement.</x:v>
+        <x:v>26 octobre 2026 : composants réels, progression préparée et fins injectées ; matériel physique, compte cloud et recette complète restent ouverts.</x:v>
       </x:c>
       <x:c r="B41" s="2"/>
       <x:c r="C41" s="2"/>
@@ -2588,14 +2588,15 @@
       </x:c>
       <x:c r="G18" s="21" t="str">
         <x:f>IF(T18&lt;&gt;"Non réalisé",T18,IF(E18=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")=E18,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H18" s="21" t="str">
         <x:v>La cité bénéficie déjà d’une session dédiée qui masque la navigation générale. Elle conserve cependant des colonnes explicatives et une scène encadrée dans une coque centrée, plutôt qu’un environnement occupant tout l’écran.</x:v>
       </x:c>
       <x:c r="I18" s="21" t="str">
         <x:v>HUB-03 — Cité rendue dans une scène fixe couvrant le viewport : lieu courant, interaction, mini-carte et objectif restent contextuels.
-HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.</x:v>
+HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.
+Suite du 26/10 : les habitants gardent leurs positions lors des réaffichages équivalents du parent. Le terminal annule le trajet et les entrées ; déplacement maintenu indépendant par touche/pointeur. Reprise après erreur sans téléporter l’Ancre ; cadrage de mini-carte borné au quartier.</x:v>
       </x:c>
       <x:c r="J18" s="21" t="str">
         <x:v>Conserver déplacements clavier et tactiles, interactions, quartiers, raccourcis et informations. Le ratio du canvas est protégé par ses styles importés : ne pas conclure à un étirement certain sans mesure.</x:v>
@@ -2609,7 +2610,8 @@
 La position est sauvegardée à un point de contrôle toutes les cinq secondes ; une fermeture brutale peut perdre les dernières secondes de marche.
 La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
 Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.</x:v>
+Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
+Quartier Atrium et équipe préparée ; aucun nouveau décor généré, pas de recette exhaustive de tous les quartiers ou de leurs services.</x:v>
       </x:c>
       <x:c r="M18" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2620,7 +2622,8 @@
 scripts/mosaicCityRuntime.test.mjs
 scripts/immersiveHubState.test.mjs
 src/components/RaceMode.jsx
-scripts/nonCombatTrial.test.mjs</x:v>
+scripts/nonCombatTrial.test.mjs
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="N18" s="21" t="str">
         <x:v>HUB-03, HUB-12</x:v>
@@ -2644,10 +2647,10 @@
         <x:v>Donner le viewport à l’exploration. Placer uniquement quartier, objectif court, minimap, interaction et pause dans le HUD ; ouvrir le journal, les statistiques et les destinations depuis une tablette ou une borne.</x:v>
       </x:c>
       <x:c r="S18" s="21" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>Cité : déplacement au clavier, deux contacts simulés, terminal, pause, réaffichage, position après remontage, récupération après erreur ; quatre formats et FR/EN. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T18" s="21" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="181" customHeight="1">
@@ -2674,14 +2677,15 @@
       </x:c>
       <x:c r="G19" s="22" t="str">
         <x:f>IF(T19&lt;&gt;"Non réalisé",T19,IF(E19=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")=E19,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-03",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H19" s="22" t="str">
         <x:v>L’exploration affiche plusieurs blocs d’accueil et de guide ainsi que des relectures. L’atlas des destinations dispose déjà de recherche et pagination. Certaines zones de service nommées n’ont pas d’action reliée dans leurs définitions.</x:v>
       </x:c>
       <x:c r="I19" s="22" t="str">
         <x:v>HUB-03 — Cité rendue dans une scène fixe couvrant le viewport : lieu courant, interaction, mini-carte et objectif restent contextuels.
-HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.</x:v>
+HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.
+Suite du 26/10 : les habitants gardent leurs positions lors des réaffichages équivalents du parent. Le terminal annule le trajet et les entrées ; déplacement maintenu indépendant par touche/pointeur. Reprise après erreur sans téléporter l’Ancre ; cadrage de mini-carte borné au quartier.</x:v>
       </x:c>
       <x:c r="J19" s="22" t="str">
         <x:v>Conserver tous les tutoriels, destinations, descriptions et raccourcis. Le passage Cité vers Missions ou Codex transmet déjà l’univers ; préserver cette amélioration au lieu de la présenter comme absente.</x:v>
@@ -2695,7 +2699,8 @@
 La position est sauvegardée à un point de contrôle toutes les cinq secondes ; une fermeture brutale peut perdre les dernières secondes de marche.
 La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
 Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.</x:v>
+Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
+Quartier Atrium et équipe préparée ; aucun nouveau décor généré, pas de recette exhaustive de tous les quartiers ou de leurs services.</x:v>
       </x:c>
       <x:c r="M19" s="22" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2706,7 +2711,8 @@
 scripts/mosaicCityRuntime.test.mjs
 scripts/immersiveHubState.test.mjs
 src/components/RaceMode.jsx
-scripts/nonCombatTrial.test.mjs</x:v>
+scripts/nonCombatTrial.test.mjs
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="N19" s="22" t="str">
         <x:v>HUB-03, HUB-12</x:v>
@@ -2729,10 +2735,10 @@
         <x:v>Montrer une transmission ou une tâche tutorielle à la fois, puis ranger sa relecture dans Aide. Ouvrir l’atlas à la demande et relier les services aux écrans existants lorsque leur fonction est disponible.</x:v>
       </x:c>
       <x:c r="S19" s="22" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>Cité : déplacement au clavier, deux contacts simulés, terminal, pause, réaffichage, position après remontage, récupération après erreur ; quatre formats et FR/EN. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T19" s="22" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="51" customHeight="1">
@@ -2759,13 +2765,14 @@
       </x:c>
       <x:c r="G20" s="21" t="str">
         <x:f>IF(T20&lt;&gt;"Non réalisé",T20,IF(E20=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Observé sur branche")=E20,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H20" s="21" t="str">
         <x:v>La préparation propose déjà les variantes de mode, le héros, une description et le rôle avant lancement. La forme actuelle repose surtout sur des sélecteurs et des explications regroupés dans un panneau.</x:v>
       </x:c>
       <x:c r="I20" s="21" t="str">
-        <x:v>HUB-04 — Préparation Extinction avec quatre cartes de variantes, aperçu de la signature et carrière XP/runs/victoires.</x:v>
+        <x:v>HUB-04 — Préparation Extinction avec quatre cartes de variantes, aperçu de la signature et carrière XP/runs/victoires.
+Suite du 26/10 : une touche relâchée ne coupe plus un autre contrôle maintenu. Visée par pointeur propriétaire et seuil cumulé de glissement ; commandes tactiles capturées. Directive · Commandes suspend la simulation. HUD compact et contrôles adaptés au paysage court. Panne de rendu récupérable sans victoire.</x:v>
       </x:c>
       <x:c r="J20" s="21" t="str">
         <x:v>Conserver les quatre variantes, tous les héros autorisés, les descriptions de rôle et les conditions de lancement. Ne pas remplacer les paramètres par une sélection visuelle moins complète.</x:v>
@@ -2774,12 +2781,14 @@
         <x:v>Lancer doit utiliser exactement la configuration affichée. Revenir d’une partie ou annuler doit retrouver les choix, et les contrôles doivent rester accessibles sans imposer la lecture de toute la documentation.</x:v>
       </x:c>
       <x:c r="L20" s="21" t="str">
-        <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.</x:v>
+        <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.
+Les débuts de run sont réels ; les conditions finales et fautes sont injectées. Pas de certification sur smartphone physique, compte cloud ou partie naturelle complète.</x:v>
       </x:c>
       <x:c r="M20" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
 src/components/HubImmersion.css
-src/components/useSceneViewport.js</x:v>
+src/components/useSceneViewport.js
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="N20" s="21" t="str">
         <x:v>HUB-04</x:v>
@@ -2800,10 +2809,10 @@
         <x:v>Construire une présentation de déploiement avec le héros et l’environnement dominants, les variantes sous forme de choix lisibles et les consignes dans un briefing court. La configuration détaillée peut rester dans un sous-menu.</x:v>
       </x:c>
       <x:c r="S20" s="21" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>Quatre variantes : extraction, last_signal, infestation, hunt. Clavier, contacts simulés, visée, Directive, pause, réaffichage, HUD agrandi et erreurs. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T20" s="21" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="129" customHeight="1">
@@ -2830,14 +2839,15 @@
       </x:c>
       <x:c r="G21" s="22" t="str">
         <x:f>IF(T21&lt;&gt;"Non réalisé",T21,IF(E21=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")=E21,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-04",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H21" s="22" t="str">
         <x:v>Pendant la partie, la configuration est masquée, mais statistiques, objectif et plusieurs boutons occupent encore une zone avant le canvas. Le cadre actif reste plafonné en largeur dans la session dédiée.</x:v>
       </x:c>
       <x:c r="I21" s="22" t="str">
         <x:v>HUB-04 — Préparation Extinction avec quatre cartes de variantes, aperçu de la signature et carrière XP/runs/victoires.
-HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.</x:v>
+HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.
+Suite du 26/10 : une touche relâchée ne coupe plus un autre contrôle maintenu. Visée par pointeur propriétaire et seuil cumulé de glissement ; commandes tactiles capturées. Directive · Commandes suspend la simulation. HUD compact et contrôles adaptés au paysage court. Panne de rendu récupérable sans victoire.</x:v>
       </x:c>
       <x:c r="J21" s="22" t="str">
         <x:v>Conserver tous les contrôles de tir et de déplacement, les variantes, l’état de la session et les informations nécessaires. L’interface doit rester lisible même lorsque le décor est lumineux ou chargé.</x:v>
@@ -2849,7 +2859,8 @@
         <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.
 La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
 Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.</x:v>
+Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
+Les débuts de run sont réels ; les conditions finales et fautes sont injectées. Pas de certification sur smartphone physique, compte cloud ou partie naturelle complète.</x:v>
       </x:c>
       <x:c r="M21" s="22" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2858,7 +2869,8 @@
 src/components/RaceMode.jsx
 src/game/immersiveHubState.js
 scripts/immersiveHubState.test.mjs
-scripts/nonCombatTrial.test.mjs</x:v>
+scripts/nonCombatTrial.test.mjs
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="N21" s="22" t="str">
         <x:v>HUB-04, HUB-12</x:v>
@@ -2880,10 +2892,10 @@
         <x:v>Faire de la vue FPS le fond de l’écran et y ancrer munitions, santé et objectif. Ranger les explications détaillées en pause, et placer les commandes tactiles près des zones d’usage selon le périphérique.</x:v>
       </x:c>
       <x:c r="S21" s="22" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>Quatre variantes : extraction, last_signal, infestation, hunt. Clavier, contacts simulés, visée, Directive, pause, réaffichage, HUD agrandi et erreurs. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T21" s="22" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="142" customHeight="1">
@@ -2910,14 +2922,15 @@
       </x:c>
       <x:c r="G22" s="21" t="str">
         <x:f>IF(T22&lt;&gt;"Non réalisé",T22,IF(E22=0,"Non réalisé",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-05",Actions!$F$7:$F$45,"Échec")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Échec")&gt;0,"Échec",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-05",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")=E22,"Observé sur branche",IF(COUNTIFS(Actions!$A$7:$A$45,"HUB-05",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Observé sur branche")+COUNTIFS(Actions!$A$7:$A$45,"HUB-05",Actions!$F$7:$F$45,"Partiel")+COUNTIFS(Actions!$A$7:$A$45,"HUB-12",Actions!$F$7:$F$45,"Partiel")&gt;0,"Partiel","Non réalisé")))))</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="H22" s="21" t="str">
         <x:v>La fin de session transmet un rapport contenant résultat et récompenses. Le callback parent récupéré ferme la session sans exploiter ce rapport, alors que le bilan annonce des gains d’or, fragments et expérience.</x:v>
       </x:c>
       <x:c r="I22" s="21" t="str">
         <x:v>HUB-05 — Chaque run reçoit un identifiant unique. Le rapport de verdict est consommé par setGold, setBreachShards et setActivityProgress.
-HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.</x:v>
+HUB-12 — Revue de code après premier commit : les jauges et les dix commandes Extinction partagent désormais un quai à hauteur naturelle. Même principe pour la cache Course et ses commandes ; leur retour à la ligne ne provoque plus de chevauchement lié à des offsets fixes.
+Suite du 26/10 : bilan modal avec focus sur Continuer, arrière-plan inerte et Échap sans abandon du verdict. Fin autorisée uniquement depuis un run actif ; signal doublé ignoré. L’économie et le callback de progression existants sont conservés.</x:v>
       </x:c>
       <x:c r="J22" s="21" t="str">
         <x:v>Conserver le rapport, ses scores, son résultat et ses gains prévus. Ne pas ajouter une deuxième attribution lors de la fermeture, de la reprise ou de l’affichage du résultat.</x:v>
@@ -2930,7 +2943,8 @@
 Une victoire jouée de bout en bout dans chaque variante reste à vérifier en preview. La preuve actuelle couvre le callback réel et la simulation déterministe.
 La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
 Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.</x:v>
+Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
+Les rapports de fin des parcours navigateur proviennent de conditions terminales injectées, pas de victoires jouées intégralement.</x:v>
       </x:c>
       <x:c r="M22" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2939,7 +2953,8 @@
 src/components/RaceMode.jsx
 src/components/HubImmersion.css
 src/components/useSceneViewport.js
-scripts/nonCombatTrial.test.mjs</x:v>
+scripts/nonCombatTrial.test.mjs
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="N22" s="21" t="str">
         <x:v>HUB-05, HUB-12</x:v>
@@ -2961,10 +2976,10 @@
         <x:v>Vérifier ce chemin par une victoire contrôlée puis raccorder le bilan à la progression, ou expliciter un résultat de simulation si aucun gain ne doit être attribué. Présenter ensuite le bilan dans la scène avec une sortie volontaire.</x:v>
       </x:c>
       <x:c r="S22" s="21" t="str">
-        <x:v>Aucune observation de la nouvelle branche enregistrée.</x:v>
+        <x:v>Bilan des quatre variantes, navigation Tab, fermeture explicite et callback de fin unique ; aucune récompense sur erreur de rendu. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T22" s="21" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="77" customHeight="1">
@@ -4946,7 +4961,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R329e0c628dc54133"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea0e885a010d4720"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5852,7 +5867,7 @@
         <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F20" s="23" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G20" s="21" t="str">
         <x:v>Cité rendue dans une scène fixe couvrant le viewport : lieu courant, interaction, mini-carte et objectif restent contextuels.
@@ -5860,7 +5875,8 @@
 Destinations, statistiques, journal, commandes et gestion du guide sont déplacés dans un terminal ouvrable qui gèle l’exploration.
 Un seul panneau de guide est affiché : dialogue d’accueil ou étape active. Pause, reprise, ignorer, redémarrer et revoir l’accueil restent disponibles.
 Position, orientation et quartier sont sauvegardés dans activityProgress.mosaicLocation toutes les cinq secondes, à la sortie et au pagehide. Retour sûr à l’Atrium si le quartier devient indisponible.
-Services connectés : Archives → Codex ; chambre des arcs → arcs ; relectures → journal ; récupération → équipe ; reliques → inventaire ; simulateur → Custom. La navigation mission conserve le contexte de l’univers malgré la remise à zéro des sous-vues.</x:v>
+Services connectés : Archives → Codex ; chambre des arcs → arcs ; relectures → journal ; récupération → équipe ; reliques → inventaire ; simulateur → Custom. La navigation mission conserve le contexte de l’univers malgré la remise à zéro des sous-vues.
+Suite du 26/10 : les habitants gardent leurs positions lors des réaffichages équivalents du parent. Le terminal annule le trajet et les entrées ; déplacement maintenu indépendant par touche/pointeur. Reprise après erreur sans téléporter l’Ancre ; cadrage de mini-carte borné au quartier.</x:v>
       </x:c>
       <x:c r="H20" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -5869,22 +5885,26 @@
 src/components/ImmersiveDrawer.jsx
 src/game/immersiveHubState.js
 scripts/mosaicCityRuntime.test.mjs
-scripts/immersiveHubState.test.mjs</x:v>
+scripts/immersiveHubState.test.mjs
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="I20" s="21" t="str">
         <x:v>34 tests mosaicCityRuntime réussis, dont navigation de proximité, destinations autorisées, tutoriel, collisions et entrées clavier/tactiles.
 Tests nouveaux : déplacement réel puis sérialisation/restauration du quartier/position ; limites et données invalides ; état transitoire non sauvegardé.
 Oxlint sur les six sources du lot : succès, aucun avertissement.
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
-git diff --check : succès.</x:v>
+git diff --check : succès.
+26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
+Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
       </x:c>
       <x:c r="J20" s="21" t="str">
         <x:v>Les portails restent soumis à proximité et autorisation ; le terminal ne téléporte pas dans un univers verrouillé.
 Le décor illustré ajouté réutilise uniquement l’Atrium existant. Les autres quartiers gardent leur décor procédural.
-La position est sauvegardée à un point de contrôle toutes les cinq secondes ; une fermeture brutale peut perdre les dernières secondes de marche.</x:v>
+La position est sauvegardée à un point de contrôle toutes les cinq secondes ; une fermeture brutale peut perdre les dernières secondes de marche.
+Quartier Atrium et équipe préparée ; aucun nouveau décor généré, pas de recette exhaustive de tous les quartiers ou de leurs services.</x:v>
       </x:c>
       <x:c r="K20" s="21" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>Cité : déplacement au clavier, deux contacts simulés, terminal, pause, réaffichage, position après remontage, récupération après erreur ; quatre formats et FR/EN. Preuves : https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="L20" s="27" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -5918,29 +5938,34 @@
         <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G21" s="22" t="str">
         <x:v>Préparation Extinction avec quatre cartes de variantes, aperçu de la signature et carrière XP/runs/victoires.
 Partie FPS dans une scène couvrant le viewport, avec objectif, PV/armure/munitions et commandes superposés aux bords. Radar, réticule, arme et simulation sont conservés.
-Suppression du doublon visuel des mêmes statistiques dans le canevas, puisque toutes restent présentes dans un HUD DOM lisible et accessible.</x:v>
+Suppression du doublon visuel des mêmes statistiques dans le canevas, puisque toutes restent présentes dans un HUD DOM lisible et accessible.
+Suite du 26/10 : une touche relâchée ne coupe plus un autre contrôle maintenu. Visée par pointeur propriétaire et seuil cumulé de glissement ; commandes tactiles capturées. Directive · Commandes suspend la simulation. HUD compact et contrôles adaptés au paysage court. Panne de rendu récupérable sans victoire.</x:v>
       </x:c>
       <x:c r="H21" s="22" t="str">
         <x:v>src/components/HubScreen.jsx
 src/components/HubImmersion.css
-src/components/useSceneViewport.js</x:v>
+src/components/useSceneViewport.js
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="I21" s="22" t="str">
         <x:v>extinctionTiming : simulation réelle, dégâts, déplacements et recharge identiques à 30/60/120/144 Hz ; pause et visibilité sans rattrapage.
 Oxlint sur les six sources du lot : succès, aucun avertissement.
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
-git diff --check : succès.</x:v>
+git diff --check : succès.
+26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
+Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
       </x:c>
       <x:c r="J21" s="22" t="str">
-        <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.</x:v>
+        <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.
+Les débuts de run sont réels ; les conditions finales et fautes sont injectées. Pas de certification sur smartphone physique, compte cloud ou partie naturelle complète.</x:v>
       </x:c>
       <x:c r="K21" s="22" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>Quatre variantes : extraction, last_signal, infestation, hunt. Clavier, contacts simulés, visée, Directive, pause, réaffichage, HUD agrandi et erreurs. Preuves : https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="L21" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -5974,32 +5999,37 @@
         <x:v>Réussis</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G22" s="21" t="str">
         <x:v>Chaque run reçoit un identifiant unique. Le rapport de verdict est consommé par setGold, setBreachShards et setActivityProgress.
 Or et fragments affichés sont transférés aux compteurs réels. XP Extinction sauvegardée dans extinctionCareer, avec nombre de runs, victoires, reçu et dernier rapport ; journal conservé.
 Le reçu empêche un versement répété. Abandon et rapport mal formé ne donnent pas de récompense. Les gains de repli du moteur sont respectés.
-Le résultat demeure en scène dédiée jusqu’à Continuer ; sa validation ne verse rien une seconde fois.</x:v>
+Le résultat demeure en scène dédiée jusqu’à Continuer ; sa validation ne verse rien une seconde fois.
+Suite du 26/10 : bilan modal avec focus sur Continuer, arrière-plan inerte et Échap sans abandon du verdict. Fin autorisée uniquement depuis un run actif ; signal doublé ignoré. L’économie et le callback de progression existants sont conservés.</x:v>
       </x:c>
       <x:c r="H22" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
 src/game/immersiveHubState.js
-scripts/immersiveHubState.test.mjs</x:v>
+scripts/immersiveHubState.test.mjs
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
       </x:c>
       <x:c r="I22" s="21" t="str">
         <x:v>Exécution du vrai callback Hub dans le test : +172 Or / +45 fragments / +210 XP une seule fois sur double rapport ; aucun appel de sortie avant acknowledgement ; bilan défaite distinct.
 Sérialisation/rechargement du reçu : même rapport refusé ; données de progression sans rapport conservées.
 Oxlint sur les six sources du lot : succès, aucun avertissement.
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
-git diff --check : succès.</x:v>
+git diff --check : succès.
+26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
+Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
       </x:c>
       <x:c r="J22" s="21" t="str">
         <x:v>Les gains sont ceux du moteur existant ; aucune révision économique ajoutée.
-Une victoire jouée de bout en bout dans chaque variante reste à vérifier en preview. La preuve actuelle couvre le callback réel et la simulation déterministe.</x:v>
+Une victoire jouée de bout en bout dans chaque variante reste à vérifier en preview. La preuve actuelle couvre le callback réel et la simulation déterministe.
+Les rapports de fin des parcours navigateur proviennent de conditions terminales injectées, pas de victoires jouées intégralement.</x:v>
       </x:c>
       <x:c r="K22" s="21" t="str">
-        <x:v>Aucune preuve navigateur de la branche enregistrée.</x:v>
+        <x:v>Bilan des quatre variantes, navigation Tab, fermeture explicite et callback de fin unique ; aucune récompense sur erreur de rendu. Preuves : https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="L22" s="27" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -7350,7 +7380,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f20f6069fb408d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38a2584b51564768"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7787,7 +7817,7 @@
       </x:c>
       <x:c r="F18" s="21" t="str">
         <x:f>'40 écrans'!G18</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G18" s="21" t="str">
         <x:v>Le monde doit rester visible sans défilement pour atteindre une action. Changer de taille doit préserver ratio et coordonnées d’interaction, et revenir d’un dossier doit retrouver le quartier et la position utiles.</x:v>
@@ -7816,7 +7846,7 @@
       </x:c>
       <x:c r="F19" s="22" t="str">
         <x:f>'40 écrans'!G19</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G19" s="22" t="str">
         <x:v>Chaque borne doit mener à une fonction réelle ou expliquer son état. Retourner au monde doit conserver le point de reprise, et fermer une aide ne doit pas désactiver la progression tutorielle.</x:v>
@@ -7845,7 +7875,7 @@
       </x:c>
       <x:c r="F20" s="21" t="str">
         <x:f>'40 écrans'!G20</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G20" s="21" t="str">
         <x:v>Lancer doit utiliser exactement la configuration affichée. Revenir d’une partie ou annuler doit retrouver les choix, et les contrôles doivent rester accessibles sans imposer la lecture de toute la documentation.</x:v>
@@ -7874,7 +7904,7 @@
       </x:c>
       <x:c r="F21" s="22" t="str">
         <x:f>'40 écrans'!G21</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G21" s="22" t="str">
         <x:v>Aucune commande indispensable ne doit demander de faire défiler la page pendant le tir. Pause, reprise et changement de visibilité doivent conserver la session et éviter les entrées maintenues involontaires.</x:v>
@@ -7903,7 +7933,7 @@
       </x:c>
       <x:c r="F22" s="21" t="str">
         <x:f>'40 écrans'!G22</x:f>
-        <x:v>Non réalisé</x:v>
+        <x:v>Partiel</x:v>
       </x:c>
       <x:c r="G22" s="21" t="str">
         <x:v>Les valeurs avant et après une victoire doivent correspondre aux gains affichés. Revoir ou fermer le bilan ne doit pas les multiplier ; un abandon ne doit pas être traité comme une victoire.</x:v>
@@ -8632,7 +8662,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07df8ff7298241bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R289ba408adab441e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11628,6 +11658,370 @@
         <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/race-continuation-2026-10-26.json</x:v>
       </x:c>
       <x:c r="H124" s="50" t="str">
+        <x:v>Périmètre de livraison</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="118" customHeight="1">
+      <x:c r="A125" s="49" t="str">
+        <x:v>SCENES-BASELINE</x:v>
+      </x:c>
+      <x:c r="B125" s="49" t="str">
+        <x:v>Historique CI</x:v>
+      </x:c>
+      <x:c r="C125" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D125" s="49" t="str">
+        <x:v>Commit c10f75b</x:v>
+      </x:c>
+      <x:c r="E125" s="49" t="str">
+        <x:v>Les quatre workflows de référence sont réussis : Course, fiabilité, signatures et build complet.</x:v>
+      </x:c>
+      <x:c r="F125" s="49" t="str">
+        <x:v>Résultats de la version précédente, pas du nouveau commit.</x:v>
+      </x:c>
+      <x:c r="G125" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40275358402</x:v>
+      </x:c>
+      <x:c r="H125" s="49" t="str">
+        <x:v>GitHub Actions, contrôle du 26/10/2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="118" customHeight="1">
+      <x:c r="A126" s="49" t="str">
+        <x:v>SCENES-INPUT</x:v>
+      </x:c>
+      <x:c r="B126" s="49" t="str">
+        <x:v>Correction et régression</x:v>
+      </x:c>
+      <x:c r="C126" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D126" s="49" t="str">
+        <x:v>Clavier et pointeurs indépendants</x:v>
+      </x:c>
+      <x:c r="E126" s="49" t="str">
+        <x:v>Relâcher W ne libère pas ArrowUp ni un bouton tactile encore maintenu. Capture, annulation, perte de capture et démontage nettoient leur propre source.</x:v>
+      </x:c>
+      <x:c r="F126" s="49" t="str">
+        <x:v>Contacts simulés dans Chromium ; matériel tactile physique non testé.</x:v>
+      </x:c>
+      <x:c r="G126" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H126" s="49" t="str">
+        <x:v>sceneInputs.test.mjs ; browserCityExtinction.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="118" customHeight="1">
+      <x:c r="A127" s="49" t="str">
+        <x:v>SCENES-UNIT</x:v>
+      </x:c>
+      <x:c r="B127" s="49" t="str">
+        <x:v>Tests unitaires</x:v>
+      </x:c>
+      <x:c r="C127" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D127" s="49" t="str">
+        <x:v>Scènes, horloge, entrées, progression</x:v>
+      </x:c>
+      <x:c r="E127" s="49" t="str">
+        <x:v>64/64 réussis, dont 14 nouveaux tests d’entrées et contrats Cité/Extinction.</x:v>
+      </x:c>
+      <x:c r="F127" s="49" t="str">
+        <x:v>La suite contient des contrôles présents dans la suite UI ; ne pas additionner comme tests uniques.</x:v>
+      </x:c>
+      <x:c r="G127" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H127" s="49" t="str">
+        <x:v>unit.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="118" customHeight="1">
+      <x:c r="A128" s="49" t="str">
+        <x:v>SCENES-UI</x:v>
+      </x:c>
+      <x:c r="B128" s="49" t="str">
+        <x:v>Non-régression UI</x:v>
+      </x:c>
+      <x:c r="C128" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D128" s="49" t="str">
+        <x:v>Suite immersive existante</x:v>
+      </x:c>
+      <x:c r="E128" s="49" t="str">
+        <x:v>68/68 réussis sur les sources de cette reprise.</x:v>
+      </x:c>
+      <x:c r="F128" s="49" t="str">
+        <x:v>Les autres modes ne sont pas tous parcourus visuellement par cette suite.</x:v>
+      </x:c>
+      <x:c r="G128" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H128" s="49" t="str">
+        <x:v>ui-contracts.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="118" customHeight="1">
+      <x:c r="A129" s="49" t="str">
+        <x:v>SCENES-LINT</x:v>
+      </x:c>
+      <x:c r="B129" s="49" t="str">
+        <x:v>Analyse statique</x:v>
+      </x:c>
+      <x:c r="C129" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D129" s="49" t="str">
+        <x:v>Sept sources et tests</x:v>
+      </x:c>
+      <x:c r="E129" s="49" t="str">
+        <x:v>Oxlint avec --max-warnings 0 : zéro erreur et zéro avertissement.</x:v>
+      </x:c>
+      <x:c r="F129" s="49" t="str">
+        <x:v>N’inclut pas une analyse de toute la base.</x:v>
+      </x:c>
+      <x:c r="G129" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H129" s="49" t="str">
+        <x:v>lint.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="118" customHeight="1">
+      <x:c r="A130" s="49" t="str">
+        <x:v>SCENES-BUILD</x:v>
+      </x:c>
+      <x:c r="B130" s="49" t="str">
+        <x:v>Compilation</x:v>
+      </x:c>
+      <x:c r="C130" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D130" s="49" t="str">
+        <x:v>Snapshot source</x:v>
+      </x:c>
+      <x:c r="E130" s="49" t="str">
+        <x:v>Compilation Vite réussie ; code de la Cité et d’Extinction inclus.</x:v>
+      </x:c>
+      <x:c r="F130" s="49" t="str">
+        <x:v>Checkout partiel et avertissement de taille de bundle existant ; ce n’est pas le build de production avec tous les médias.</x:v>
+      </x:c>
+      <x:c r="G130" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H130" s="49" t="str">
+        <x:v>source-build.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="118" customHeight="1">
+      <x:c r="A131" s="49" t="str">
+        <x:v>SCENES-BROWSER</x:v>
+      </x:c>
+      <x:c r="B131" s="49" t="str">
+        <x:v>Navigateur avec médias</x:v>
+      </x:c>
+      <x:c r="C131" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D131" s="49" t="str">
+        <x:v>Dix parcours Chromium</x:v>
+      </x:c>
+      <x:c r="E131" s="49" t="str">
+        <x:v>10/10 réussis avec les vrais composants et images du dépôt, quatre formats (390 à 2560 px), français/anglais.</x:v>
+      </x:c>
+      <x:c r="F131" s="49" t="str">
+        <x:v>Profil et équipe préparés ; fins et erreurs injectées. Ce ne sont pas dix parties naturelles complètes.</x:v>
+      </x:c>
+      <x:c r="G131" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H131" s="49" t="str">
+        <x:v>browser/results.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="145" customHeight="1">
+      <x:c r="A132" s="49" t="str">
+        <x:v>CITE-RETURNS</x:v>
+      </x:c>
+      <x:c r="B132" s="49" t="str">
+        <x:v>Conservation de session</x:v>
+      </x:c>
+      <x:c r="C132" s="49" t="str">
+        <x:v>Partiel</x:v>
+      </x:c>
+      <x:c r="D132" s="49" t="str">
+        <x:v>Cité-Mosaïque / Atrium</x:v>
+      </x:c>
+      <x:c r="E132" s="49" t="str">
+        <x:v>Déplacement, contacts indépendants, terminal, route annulée, pause, réaffichage sans déplacer les PNJ et position restaurée après remontage.</x:v>
+      </x:c>
+      <x:c r="F132" s="49" t="str">
+        <x:v>Les services et les quartiers autres que l’Atrium restent à parcourir intégralement.</x:v>
+      </x:c>
+      <x:c r="G132" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H132" s="49" t="str">
+        <x:v>city-*-lifecycle ; browser/results.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="145" customHeight="1">
+      <x:c r="A133" s="49" t="str">
+        <x:v>EXT-4MODES</x:v>
+      </x:c>
+      <x:c r="B133" s="49" t="str">
+        <x:v>Parcours de variantes</x:v>
+      </x:c>
+      <x:c r="C133" s="49" t="str">
+        <x:v>Partiel</x:v>
+      </x:c>
+      <x:c r="D133" s="49" t="str">
+        <x:v>Extraction, dernier signal, infestation, chasse</x:v>
+      </x:c>
+      <x:c r="E133" s="49" t="str">
+        <x:v>Entrées, visée lente sans tir involontaire, Directive, pause, HUD agrandi et conditions de victoire des quatre variantes.</x:v>
+      </x:c>
+      <x:c r="F133" s="49" t="str">
+        <x:v>Conditions de fin injectées ; équilibrage et progression naturelle non certifiés.</x:v>
+      </x:c>
+      <x:c r="G133" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H133" s="49" t="str">
+        <x:v>fps-*-lifecycle ; browser/results.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="145" customHeight="1">
+      <x:c r="A134" s="49" t="str">
+        <x:v>EXT-RESULTS</x:v>
+      </x:c>
+      <x:c r="B134" s="49" t="str">
+        <x:v>Bilan et conservation</x:v>
+      </x:c>
+      <x:c r="C134" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D134" s="49" t="str">
+        <x:v>Modalité et fin unique</x:v>
+      </x:c>
+      <x:c r="E134" s="49" t="str">
+        <x:v>Le bilan garde le focus, Échap ne supprime pas le résultat, Continuer produit une seule validation. Le callback de récompense existant est conservé.</x:v>
+      </x:c>
+      <x:c r="F134" s="49" t="str">
+        <x:v>Le navigateur utilise un collecteur de rapports ; l’économie et le vrai compte sont couverts séparément / restent à vérifier en intégration.</x:v>
+      </x:c>
+      <x:c r="G134" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H134" s="49" t="str">
+        <x:v>browserCityExtinction.py ; immersiveHubState.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="118" customHeight="1">
+      <x:c r="A135" s="49" t="str">
+        <x:v>SCENES-ERRORS</x:v>
+      </x:c>
+      <x:c r="B135" s="49" t="str">
+        <x:v>Erreurs injectées</x:v>
+      </x:c>
+      <x:c r="C135" s="49" t="str">
+        <x:v>Réussis</x:v>
+      </x:c>
+      <x:c r="D135" s="49" t="str">
+        <x:v>Cité et Extinction</x:v>
+      </x:c>
+      <x:c r="E135" s="49" t="str">
+        <x:v>Deux pannes de rendu déclenchées volontairement : aucun faux résultat, récupération Cité sans téléportation, retour Extinction à la préparation.</x:v>
+      </x:c>
+      <x:c r="F135" s="49" t="str">
+        <x:v>Pannes contrôlées ; pas de garantie contre toutes les erreurs graphiques possibles.</x:v>
+      </x:c>
+      <x:c r="G135" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H135" s="49" t="str">
+        <x:v>city-390x844-fr-fault ; fps-844x390-en-fault</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="145" customHeight="1">
+      <x:c r="A136" s="49" t="str">
+        <x:v>SCENES-VISUAL</x:v>
+      </x:c>
+      <x:c r="B136" s="49" t="str">
+        <x:v>Inspection de captures</x:v>
+      </x:c>
+      <x:c r="C136" s="49" t="str">
+        <x:v>Partiel</x:v>
+      </x:c>
+      <x:c r="D136" s="49" t="str">
+        <x:v>Portrait 390×844 et bilan 844×390</x:v>
+      </x:c>
+      <x:c r="E136" s="49" t="str">
+        <x:v>Captures revues avec décor Atrium et fond FPS réels ; commandes accessibles et bilan lisible. L’en-tête QA est propre au banc de test.</x:v>
+      </x:c>
+      <x:c r="F136" s="49" t="str">
+        <x:v>L’aperçu du journal Cité reste tronqué à HUD 1,4 (texte intégral dans le terminal). Sprites d’ennemis FPS génériques, certains libellés et autres quartiers restent à améliorer.</x:v>
+      </x:c>
+      <x:c r="G136" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+      </x:c>
+      <x:c r="H136" s="49" t="str">
+        <x:v>city-390x844-en-lifecycle-city.png ; fps-390x844-en-lifecycle-run.png ; fps-844x390-fr-lifecycle-result.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="118" customHeight="1">
+      <x:c r="A137" s="49" t="str">
+        <x:v>SCENES-CI</x:v>
+      </x:c>
+      <x:c r="B137" s="49" t="str">
+        <x:v>Automatisation permanente</x:v>
+      </x:c>
+      <x:c r="C137" s="49" t="str">
+        <x:v>Déclarés</x:v>
+      </x:c>
+      <x:c r="D137" s="49" t="str">
+        <x:v>Workflow City and Extinction immersive UI</x:v>
+      </x:c>
+      <x:c r="E137" s="49" t="str">
+        <x:v>Suite dédiée ajoutée aux changements de la PR ; exige le décodage du décor de chaque scène. La vérification préalable 40279377677 est réussie.</x:v>
+      </x:c>
+      <x:c r="F137" s="49" t="str">
+        <x:v>Le workflow de la branche finale est déclenché après publication ; son état n’est pas anticipé.</x:v>
+      </x:c>
+      <x:c r="G137" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/pull/9/checks</x:v>
+      </x:c>
+      <x:c r="H137" s="49" t="str">
+        <x:v>.github/workflows/city-extinction-ui.yml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="145" customHeight="1">
+      <x:c r="A138" s="49" t="str">
+        <x:v>SCENES-LIMITES</x:v>
+      </x:c>
+      <x:c r="B138" s="49" t="str">
+        <x:v>Recette restant à réaliser</x:v>
+      </x:c>
+      <x:c r="C138" s="49" t="str">
+        <x:v>Non réalisés</x:v>
+      </x:c>
+      <x:c r="D138" s="49" t="str">
+        <x:v>Matériel / compte / 40 écrans</x:v>
+      </x:c>
+      <x:c r="E138" s="49" t="str">
+        <x:v>Manette physique, multitouch sur appareil réel, compte cloud réel, services/quartiers complets, progression intégrale et recette artistique consolidée.</x:v>
+      </x:c>
+      <x:c r="F138" s="49" t="str">
+        <x:v>Aucun de ces points n’est marqué terminé par les essais isolés.</x:v>
+      </x:c>
+      <x:c r="G138" s="49" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H138" s="49" t="str">
         <x:v>Périmètre de livraison</x:v>
       </x:c>
     </x:row>
@@ -11659,7 +12053,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c8a79faed344ad3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7f13efc895044e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): finish city journal and service continuity, localize scene objectives
Publish sixteen exact files verified by 81 targeted tests, 68 overlapping UI tests, ten lifecycle scenarios and eight new service/full-run Chromium checks. Include 144-entry Excel and CI receipt. Keep all modes and content; remove temporary source/transport workflows.
</commit_message>
<xml_diff>
--- a/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
+++ b/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Rfdf25aa27a084d81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Rd9968c246a79403f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="R109e97c4eb404e79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="Ra05bd74ebf314381"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="R326bc93759ed4779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Ra66e7982a0454dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="R42ab32bf09e24aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="R63fa9931639b4299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R70aac3a595cf4685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="R93fc1939b7244690"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -71,6 +71,17 @@
       <x:sz val="10"/>
       <x:color rgb="FF5D6878"/>
       <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF23364C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1E5661"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="6">
@@ -135,7 +146,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -281,6 +292,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -638,8 +655,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H138" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:H138"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H150" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:H150"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Réf."/>
     <x:tableColumn id="2" name="Nature de preuve"/>
@@ -896,7 +913,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>Suivi continu de l’audit des 40 écrans — suite Cité et Extinction du 26 octobre 2026.</x:v>
+        <x:v>Suivi continu de l’audit des 40 écrans — journal, services et parties Extinction du 26 octobre 2026.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1142,7 +1159,7 @@
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="46" t="str">
-        <x:v>Cité : déplacements, terminal, habitants et reprise. Extinction : entrées, visée, Directive, HUD, bilan modal et erreurs. Fonctions et contenus conservés.</x:v>
+        <x:v>Journal Cité ouvrable au HUD agrandi ; 36 transitions de services ; quatre variantes Extinction terminées par entrées automatisées.</x:v>
       </x:c>
       <x:c r="B16" s="2"/>
       <x:c r="C16" s="2"/>
@@ -1250,7 +1267,7 @@
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="46" t="str">
-        <x:v>Suite Cité/Extinction : 64 tests ciblés, 68 tests UI et 10 parcours Chromium réussis ; suites unitaires se recoupant. Quatre formats, FR/EN, vrais médias, fins préparées.</x:v>
+        <x:v>Suite : 81 tests ciblés, 68 tests UI (recoupements), quatre parcours Cité et quatre runs Extinction ; état distant dans Checks.</x:v>
       </x:c>
       <x:c r="B25" s="2"/>
       <x:c r="C25" s="2"/>
@@ -1376,7 +1393,7 @@
       </x:c>
       <x:c r="B35" s="2"/>
       <x:c r="C35" s="47" t="str">
-        <x:v>Base c10f75b / snapshot 80468d2 ; nouvelle preuve : city-extinction-continuation-2026-10-26.json.</x:v>
+        <x:v>Base d915220 / snapshot c7ce3caf ; preuves : scene-completion-2026-10-26.json et reçu CI lié dans la PR.</x:v>
       </x:c>
       <x:c r="D35" s="2"/>
       <x:c r="E35" s="2"/>
@@ -1419,7 +1436,7 @@
       </x:c>
       <x:c r="B38" s="2"/>
       <x:c r="C38" s="47" t="str">
-        <x:v>Actualisation artifact_tool ; historique Fighter, Course et Cité/Extinction conservé. Les seuls ledgers initiaux ne reproduisent pas les annotations des reprises.</x:v>
+        <x:v>Actualisation artifact_tool ; historique conservé ; 144 vérifications. Aucun écran déclaré entièrement validé par cette passe.</x:v>
       </x:c>
       <x:c r="D38" s="2"/>
       <x:c r="E38" s="2"/>
@@ -2605,13 +2622,7 @@
         <x:v>Le monde doit rester visible sans défilement pour atteindre une action. Changer de taille doit préserver ratio et coordonnées d’interaction, et revenir d’un dossier doit retrouver le quartier et la position utiles.</x:v>
       </x:c>
       <x:c r="L18" s="21" t="str">
-        <x:v>Les portails restent soumis à proximité et autorisation ; le terminal ne téléporte pas dans un univers verrouillé.
-Le décor illustré ajouté réutilise uniquement l’Atrium existant. Les autres quartiers gardent leur décor procédural.
-La position est sauvegardée à un point de contrôle toutes les cinq secondes ; une fermeture brutale peut perdre les dernières secondes de marche.
-La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
-Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
-Quartier Atrium et équipe préparée ; aucun nouveau décor généré, pas de recette exhaustive de tous les quartiers ou de leurs services.</x:v>
+        <x:v>Journal lisible et ouvrable au HUD 140 % dans les parcours vérifiés ; reste la visite exhaustive des quartiers, médias et profils.</x:v>
       </x:c>
       <x:c r="M18" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2647,7 +2658,7 @@
         <x:v>Donner le viewport à l’exploration. Placer uniquement quartier, objectif court, minimap, interaction et pause dans le HUD ; ouvrir le journal, les statistiques et les destinations depuis une tablette ou une borne.</x:v>
       </x:c>
       <x:c r="S18" s="21" t="str">
-        <x:v>Cité : déplacement au clavier, deux contacts simulés, terminal, pause, réaffichage, position après remontage, récupération après erreur ; quatre formats et FR/EN. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T18" s="21" t="str">
         <x:v>Partiel</x:v>
@@ -2694,13 +2705,7 @@
         <x:v>Chaque borne doit mener à une fonction réelle ou expliquer son état. Retourner au monde doit conserver le point de reprise, et fermer une aide ne doit pas désactiver la progression tutorielle.</x:v>
       </x:c>
       <x:c r="L19" s="22" t="str">
-        <x:v>Les portails restent soumis à proximité et autorisation ; le terminal ne téléporte pas dans un univers verrouillé.
-Le décor illustré ajouté réutilise uniquement l’Atrium existant. Les autres quartiers gardent leur décor procédural.
-La position est sauvegardée à un point de contrôle toutes les cinq secondes ; une fermeture brutale peut perdre les dernières secondes de marche.
-La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
-Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
-Quartier Atrium et équipe préparée ; aucun nouveau décor généré, pas de recette exhaustive de tous les quartiers ou de leurs services.</x:v>
+        <x:v>36 transitions validées depuis des positions préparées ; reste l’exploration naturelle de tous les quartiers et l’intégration des écrans destinataires réels.</x:v>
       </x:c>
       <x:c r="M19" s="22" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2735,7 +2740,7 @@
         <x:v>Montrer une transmission ou une tâche tutorielle à la fois, puis ranger sa relecture dans Aide. Ouvrir l’atlas à la demande et relier les services aux écrans existants lorsque leur fonction est disponible.</x:v>
       </x:c>
       <x:c r="S19" s="22" t="str">
-        <x:v>Cité : déplacement au clavier, deux contacts simulés, terminal, pause, réaffichage, position après remontage, récupération après erreur ; quatre formats et FR/EN. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T19" s="22" t="str">
         <x:v>Partiel</x:v>
@@ -2781,8 +2786,7 @@
         <x:v>Lancer doit utiliser exactement la configuration affichée. Revenir d’une partie ou annuler doit retrouver les choix, et les contrôles doivent rester accessibles sans imposer la lecture de toute la documentation.</x:v>
       </x:c>
       <x:c r="L20" s="21" t="str">
-        <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.
-Les débuts de run sont réels ; les conditions finales et fautes sont injectées. Pas de certification sur smartphone physique, compte cloud ou partie naturelle complète.</x:v>
+        <x:v>Briefing Infestation aligné sur 60 secondes ; autres textes de catalogues et toutes les combinaisons de signatures restent à relire.</x:v>
       </x:c>
       <x:c r="M20" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2809,7 +2813,7 @@
         <x:v>Construire une présentation de déploiement avec le héros et l’environnement dominants, les variantes sous forme de choix lisibles et les consignes dans un briefing court. La configuration détaillée peut rester dans un sous-menu.</x:v>
       </x:c>
       <x:c r="S20" s="21" t="str">
-        <x:v>Quatre variantes : extraction, last_signal, infestation, hunt. Clavier, contacts simulés, visée, Directive, pause, réaffichage, HUD agrandi et erreurs. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T20" s="21" t="str">
         <x:v>Partiel</x:v>
@@ -2856,11 +2860,7 @@
         <x:v>Aucune commande indispensable ne doit demander de faire défiler la page pendant le tir. Pause, reprise et changement de visibilité doivent conserver la session et éviter les entrées maintenues involontaires.</x:v>
       </x:c>
       <x:c r="L21" s="22" t="str">
-        <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.
-La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
-Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
-Les débuts de run sont réels ; les conditions finales et fautes sont injectées. Pas de certification sur smartphone physique, compte cloud ou partie naturelle complète.</x:v>
+        <x:v>Quatre modes terminés par bot, entrées normales et horloge virtuelle ; compte réel, périphériques physiques, intégration de carrière et équilibrage restent à valider.</x:v>
       </x:c>
       <x:c r="M21" s="22" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2892,7 +2892,7 @@
         <x:v>Faire de la vue FPS le fond de l’écran et y ancrer munitions, santé et objectif. Ranger les explications détaillées en pause, et placer les commandes tactiles près des zones d’usage selon le périphérique.</x:v>
       </x:c>
       <x:c r="S21" s="22" t="str">
-        <x:v>Quatre variantes : extraction, last_signal, infestation, hunt. Clavier, contacts simulés, visée, Directive, pause, réaffichage, HUD agrandi et erreurs. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T21" s="22" t="str">
         <x:v>Partiel</x:v>
@@ -2939,12 +2939,7 @@
         <x:v>Les valeurs avant et après une victoire doivent correspondre aux gains affichés. Revoir ou fermer le bilan ne doit pas les multiplier ; un abandon ne doit pas être traité comme une victoire.</x:v>
       </x:c>
       <x:c r="L22" s="21" t="str">
-        <x:v>Les gains sont ceux du moteur existant ; aucune révision économique ajoutée.
-Une victoire jouée de bout en bout dans chaque variante reste à vérifier en preview. La preuve actuelle couvre le callback réel et la simulation déterministe.
-La vérification des trois dimensions est une vérification mathématique des overlays dessinés et une revue de CSS ; aucun rendu navigateur des changements n’est revendiqué.
-Le texte des scènes et les jauges historiques dessinées par les autres moteurs ne deviennent pas tous vectoriels ni uniformément redimensionnables. La recette preview doit vérifier aussi les préférences agrandies.
-Le guide de Cité et les libellés longs doivent encore être contrôlés sur les faibles hauteurs de viewport.
-Les rapports de fin des parcours navigateur proviennent de conditions terminales injectées, pas de victoires jouées intégralement.</x:v>
+        <x:v>Quatre modes terminés par bot, entrées normales et horloge virtuelle ; compte réel, périphériques physiques, intégration de carrière et équilibrage restent à valider.</x:v>
       </x:c>
       <x:c r="M22" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -2976,7 +2971,7 @@
         <x:v>Vérifier ce chemin par une victoire contrôlée puis raccorder le bilan à la progression, ou expliciter un résultat de simulation si aucun gain ne doit être attribué. Présenter ensuite le bilan dans la scène avec une sortie volontaire.</x:v>
       </x:c>
       <x:c r="S22" s="21" t="str">
-        <x:v>Bilan des quatre variantes, navigation Tab, fermeture explicite et callback de fin unique ; aucune récompense sur erreur de rendu. https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T22" s="21" t="str">
         <x:v>Partiel</x:v>
@@ -3050,7 +3045,7 @@
         <x:v>Utiliser un garage ou une grille plein écran avec le kart sélectionné, Mirelle et un aperçu du circuit. Ranger les réglages complémentaires dans leurs rubriques et garder un résumé de course avant lancement.</x:v>
       </x:c>
       <x:c r="S23" s="22" t="str">
-        <x:v>26/10 : parcours Chromium isolés sur Course ; contrôle du garage, conduite, résultat et erreurs. Vrais composants, sans médias locaux ni compte réel.</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T23" s="22" t="str">
         <x:v>Partiel</x:v>
@@ -3130,7 +3125,7 @@
         <x:v>Donner toute la surface à la piste, avec classement, tour, temps, vitesse et objet dans un HUD compact. Déplacer carrière, achats, améliorations et descriptions vers la préparation ou la pause ; garder les commandes tactiles adaptées.</x:v>
       </x:c>
       <x:c r="S24" s="21" t="str">
-        <x:v>26/10 : parcours Chromium isolés sur Course ; contrôle du garage, conduite, résultat et erreurs. Vrais composants, sans médias locaux ni compte réel.</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T24" s="21" t="str">
         <x:v>Partiel</x:v>
@@ -3209,7 +3204,7 @@
         <x:v>Présenter un podium ou un bilan sur la scène, avec place, temps et gains immédiatement lisibles, puis un détail de carrière ouvrable. Mettre Rejouer, Changer de circuit et Quitter dans une zone d’action stable.</x:v>
       </x:c>
       <x:c r="S25" s="22" t="str">
-        <x:v>26/10 : parcours Chromium isolés sur Course ; contrôle du garage, conduite, résultat et erreurs. Vrais composants, sans médias locaux ni compte réel.</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="T25" s="22" t="str">
         <x:v>Partiel</x:v>
@@ -4961,7 +4956,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea0e885a010d4720"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2393ffe42bdb490e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5876,7 +5871,8 @@
 Un seul panneau de guide est affiché : dialogue d’accueil ou étape active. Pause, reprise, ignorer, redémarrer et revoir l’accueil restent disponibles.
 Position, orientation et quartier sont sauvegardés dans activityProgress.mosaicLocation toutes les cinq secondes, à la sortie et au pagehide. Retour sûr à l’Atrium si le quartier devient indisponible.
 Services connectés : Archives → Codex ; chambre des arcs → arcs ; relectures → journal ; récupération → équipe ; reliques → inventaire ; simulateur → Custom. La navigation mission conserve le contexte de l’univers malgré la remise à zéro des sous-vues.
-Suite du 26/10 : les habitants gardent leurs positions lors des réaffichages équivalents du parent. Le terminal annule le trajet et les entrées ; déplacement maintenu indépendant par touche/pointeur. Reprise après erreur sans téléporter l’Ancre ; cadrage de mini-carte borné au quartier.</x:v>
+Suite du 26/10 : les habitants gardent leurs positions lors des réaffichages équivalents du parent. Le terminal annule le trajet et les entrées ; déplacement maintenu indépendant par touche/pointeur. Reprise après erreur sans téléporter l’Ancre ; cadrage de mini-carte borné au quartier.
+Suite suivante : Transmission ouvrable directement au HUD agrandi. Snapshot explicite avant chaque sortie de service, y compris missions et codex ; commandes relâchées et menu fermé. 36 transitions contrôlées sur quatre formats.</x:v>
       </x:c>
       <x:c r="H20" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -5895,16 +5891,14 @@
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
 git diff --check : succès.
 26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
-Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677
+Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.</x:v>
       </x:c>
       <x:c r="J20" s="21" t="str">
-        <x:v>Les portails restent soumis à proximité et autorisation ; le terminal ne téléporte pas dans un univers verrouillé.
-Le décor illustré ajouté réutilise uniquement l’Atrium existant. Les autres quartiers gardent leur décor procédural.
-La position est sauvegardée à un point de contrôle toutes les cinq secondes ; une fermeture brutale peut perdre les dernières secondes de marche.
-Quartier Atrium et équipe préparée ; aucun nouveau décor généré, pas de recette exhaustive de tous les quartiers ou de leurs services.</x:v>
+        <x:v>Destinations préparées : neuf accès représentatifs, quatre tailles ; pas tous les quartiers ni les écrans de destination réels. Validation artistique globale, appareil physique et cloud non effectués.</x:v>
       </x:c>
       <x:c r="K20" s="21" t="str">
-        <x:v>Cité : déplacement au clavier, deux contacts simulés, terminal, pause, réaffichage, position après remontage, récupération après erreur ; quatre formats et FR/EN. Preuves : https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="L20" s="27" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -5944,7 +5938,8 @@
         <x:v>Préparation Extinction avec quatre cartes de variantes, aperçu de la signature et carrière XP/runs/victoires.
 Partie FPS dans une scène couvrant le viewport, avec objectif, PV/armure/munitions et commandes superposés aux bords. Radar, réticule, arme et simulation sont conservés.
 Suppression du doublon visuel des mêmes statistiques dans le canevas, puisque toutes restent présentes dans un HUD DOM lisible et accessible.
-Suite du 26/10 : une touche relâchée ne coupe plus un autre contrôle maintenu. Visée par pointeur propriétaire et seuil cumulé de glissement ; commandes tactiles capturées. Directive · Commandes suspend la simulation. HUD compact et contrôles adaptés au paysage court. Panne de rendu récupérable sans victoire.</x:v>
+Suite du 26/10 : une touche relâchée ne coupe plus un autre contrôle maintenu. Visée par pointeur propriétaire et seuil cumulé de glissement ; commandes tactiles capturées. Directive · Commandes suspend la simulation. HUD compact et contrôles adaptés au paysage court. Panne de rendu récupérable sans victoire.
+Suite suivante : objectif Infestation précise les 60 secondes existantes. Six noms ennemis et les armes ramassées suivent la langue d’interface, sans modifier les types internes. Les quatre variantes atteignent leur victoire par les entrées normales.</x:v>
       </x:c>
       <x:c r="H21" s="22" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -5958,14 +5953,14 @@
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
 git diff --check : succès.
 26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
-Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677
+Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.</x:v>
       </x:c>
       <x:c r="J21" s="22" t="str">
-        <x:v>Recette tactile et contrôle de la densité des boutons sur petits écrans encore nécessaires en preview.
-Les débuts de run sont réels ; les conditions finales et fautes sont injectées. Pas de certification sur smartphone physique, compte cloud ou partie naturelle complète.</x:v>
+        <x:v>Quatre victoires automatisées avec horloge virtuelle et un profil préparé. Pas de test humain, d’équilibrage ou de tous les héros/armes. Silhouettes génériques inchangées ; autres libellés à relire.</x:v>
       </x:c>
       <x:c r="K21" s="22" t="str">
-        <x:v>Quatre variantes : extraction, last_signal, infestation, hunt. Clavier, contacts simulés, visée, Directive, pause, réaffichage, HUD agrandi et erreurs. Preuves : https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="L21" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -6006,7 +6001,8 @@
 Or et fragments affichés sont transférés aux compteurs réels. XP Extinction sauvegardée dans extinctionCareer, avec nombre de runs, victoires, reçu et dernier rapport ; journal conservé.
 Le reçu empêche un versement répété. Abandon et rapport mal formé ne donnent pas de récompense. Les gains de repli du moteur sont respectés.
 Le résultat demeure en scène dédiée jusqu’à Continuer ; sa validation ne verse rien une seconde fois.
-Suite du 26/10 : bilan modal avec focus sur Continuer, arrière-plan inerte et Échap sans abandon du verdict. Fin autorisée uniquement depuis un run actif ; signal doublé ignoré. L’économie et le callback de progression existants sont conservés.</x:v>
+Suite du 26/10 : bilan modal avec focus sur Continuer, arrière-plan inerte et Échap sans abandon du verdict. Fin autorisée uniquement depuis un run actif ; signal doublé ignoré. L’économie et le callback de progression existants sont conservés.
+Suite suivante : quatre runs menés jusqu’au verdict sans injection de fin ; rapport et validation contrôlés. La carrière et les gains du vrai parent ne sont pas couverts par ce bot.</x:v>
       </x:c>
       <x:c r="H22" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -6021,7 +6017,8 @@
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
 git diff --check : succès.
 26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
-Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677</x:v>
+Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677
+Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.</x:v>
       </x:c>
       <x:c r="J22" s="21" t="str">
         <x:v>Les gains sont ceux du moteur existant ; aucune révision économique ajoutée.
@@ -6029,7 +6026,7 @@
 Les rapports de fin des parcours navigateur proviennent de conditions terminales injectées, pas de victoires jouées intégralement.</x:v>
       </x:c>
       <x:c r="K22" s="21" t="str">
-        <x:v>Bilan des quatre variantes, navigation Tab, fermeture explicite et callback de fin unique ; aucune récompense sur erreur de rendu. Preuves : https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/city-extinction-continuation-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="L22" s="27" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -6070,7 +6067,8 @@
 Le terminal de course suspend réellement l’horloge et vide les touches maintenues. Une amélioration met à jour le moteur existant au lieu de redémarrer une course.
 Scène de course sur tout le viewport, cadre caméra 960×540 conservé sans déformation, HUD et actions contextuelles superposés.
 Bilan conservé en scène jusqu’à Rejouer ou Changer de circuit ; les contrôles de la course derrière le bilan deviennent inertes.
-Suite du 26/10 : correction du redémarrage involontaire lors d’un rendu parent ou d’un achat garage. Revanche explicite avec nouvelle session, sans récompenser les anciens callbacks. Maintien des touches par pointeur ; relâchement hors bouton et activation clavier séparés. Écran de récupération après erreur de rendu. HUD portrait visible et agrandissable ; cache remise à zéro à la revanche.</x:v>
+Suite du 26/10 : correction du redémarrage involontaire lors d’un rendu parent ou d’un achat garage. Revanche explicite avec nouvelle session, sans récompenser les anciens callbacks. Maintien des touches par pointeur ; relâchement hors bouton et activation clavier séparés. Écran de récupération après erreur de rendu. HUD portrait visible et agrandissable ; cache remise à zéro à la revanche.
+Suite suivante : cinq familles d’objectifs localisées FR/EN dans le HUD et le canevas ; changement de langue sans recréer le moteur ni perdre le compteur.</x:v>
       </x:c>
       <x:c r="H23" s="22" t="str">
         <x:v>src/components/RaceMode.jsx
@@ -6090,13 +6088,14 @@
 Oxlint sur les six sources du lot : succès, aucun avertissement.
 11 fichiers de suites ciblées réussis le 25 octobre 2026 : immersiveHubState, extinctionTiming, mosaicCityRuntime, fixedStepClock, customBattle, fighterRaceGameplayAudit, kartCareerSave, catalogPagination, squadPreparation, ocCampaignUiProgress, anchorCustomization.
 git diff --check : succès.
-Suite Course : 40/40 tests unitaires, 6/6 parcours Chromium hors ligne ; aucun avertissement de lint sur les six modules/tests modifiés. Échec avant correction reproduit : moteur recréé par le parent et par l’achat ; corrigé avec assertions sur l’identité du moteur, le temps et le tour.</x:v>
+Suite Course : 40/40 tests unitaires, 6/6 parcours Chromium hors ligne ; aucun avertissement de lint sur les six modules/tests modifiés. Échec avant correction reproduit : moteur recréé par le parent et par l’achat ; corrigé avec assertions sur l’identité du moteur, le temps et le tour.
+Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.</x:v>
       </x:c>
       <x:c r="J23" s="22" t="str">
         <x:v>Ratio 16:9 conservé : bandes de fond possibles sans recadrage. Six parcours isolés, carrière préparée et deux erreurs injectées ; ce n’est pas une campagne complète. La télémétrie portrait est lisible dans le DOM, mais des libellés du moteur restent en français. Absence locale des médias ; contrôle des sept images requis par le nouveau workflow. Manette, multitouch réel et cloud restent non testés.</x:v>
       </x:c>
       <x:c r="K23" s="22" t="str">
-        <x:v>Capture et résultats Chromium hors ligne : race-ui-qa/browser-final ; 390×844, 844×390, 1280×900, 2560×1080. Composants réels, données et résultat préparés.</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
       </x:c>
       <x:c r="L23" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/RaceMode.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -7380,7 +7379,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38a2584b51564768"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc922c48618ae473c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8662,7 +8661,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R289ba408adab441e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd7837f16ee743d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12023,6 +12022,318 @@
       </x:c>
       <x:c r="H138" s="49" t="str">
         <x:v>Périmètre de livraison</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="72" customHeight="1">
+      <x:c r="A139" s="52" t="str">
+        <x:v>SUITE-JOURNAL</x:v>
+      </x:c>
+      <x:c r="B139" s="51" t="str">
+        <x:v>Code et navigateur local</x:v>
+      </x:c>
+      <x:c r="C139" s="51" t="str">
+        <x:v>Réussi — partiel</x:v>
+      </x:c>
+      <x:c r="D139" s="51" t="str">
+        <x:v>12, 13 / HUB-03</x:v>
+      </x:c>
+      <x:c r="E139" s="51" t="str">
+        <x:v>HUD 140 %, bouton Transmission, lecture complète, focus et retour Échap.</x:v>
+      </x:c>
+      <x:c r="F139" s="51" t="str">
+        <x:v>Replay hors ligne des composants réels avec médias exacts ; pas de compte ni téléphone physique.</x:v>
+      </x:c>
+      <x:c r="G139" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H139" s="51" t="str">
+        <x:v>src/components/HubScreen.jsx ; HubImmersion.css</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="72" customHeight="1">
+      <x:c r="A140" s="52" t="str">
+        <x:v>SUITE-SERVICES</x:v>
+      </x:c>
+      <x:c r="B140" s="51" t="str">
+        <x:v>Parcours navigateur local</x:v>
+      </x:c>
+      <x:c r="C140" s="51" t="str">
+        <x:v>36/36 transitions</x:v>
+      </x:c>
+      <x:c r="D140" s="51" t="str">
+        <x:v>13 / HUB-03</x:v>
+      </x:c>
+      <x:c r="E140" s="51" t="str">
+        <x:v>9 accès × 4 formats ; missions, codex, arcs, journal, équipe, inventaire, simulateur et deux bornes Nexus.</x:v>
+      </x:c>
+      <x:c r="F140" s="51" t="str">
+        <x:v>Points d’entrée préparés ; callbacks réels de la scène, écrans destinataires remplacés par le parent de test.</x:v>
+      </x:c>
+      <x:c r="G140" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H140" s="51" t="str">
+        <x:v>scripts/browserSceneServices.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="72" customHeight="1">
+      <x:c r="A141" s="52" t="str">
+        <x:v>SUITE-EXTRACTION</x:v>
+      </x:c>
+      <x:c r="B141" s="51" t="str">
+        <x:v>Partie par entrées automatisées</x:v>
+      </x:c>
+      <x:c r="C141" s="51" t="str">
+        <x:v>Victoire</x:v>
+      </x:c>
+      <x:c r="D141" s="51" t="str">
+        <x:v>15, 16 / HUB-04, HUB-05</x:v>
+      </x:c>
+      <x:c r="E141" s="51" t="str">
+        <x:v>Run Extraction : déplacement, tir, recharge, ramassage de 3 balises et victoire.</x:v>
+      </x:c>
+      <x:c r="F141" s="51" t="str">
+        <x:v>Profil préparé, bot en lecture seule et horloge virtuelle ; aucune fin, santé ou élimination injectée.</x:v>
+      </x:c>
+      <x:c r="G141" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H141" s="51" t="str">
+        <x:v>scripts/browserSceneServices.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="72" customHeight="1">
+      <x:c r="A142" s="52" t="str">
+        <x:v>SUITE-LAST-SIGNAL</x:v>
+      </x:c>
+      <x:c r="B142" s="51" t="str">
+        <x:v>Partie par entrées automatisées</x:v>
+      </x:c>
+      <x:c r="C142" s="51" t="str">
+        <x:v>Victoire</x:v>
+      </x:c>
+      <x:c r="D142" s="51" t="str">
+        <x:v>15, 16 / HUB-04, HUB-05</x:v>
+      </x:c>
+      <x:c r="E142" s="51" t="str">
+        <x:v>Run Dernier Signal : vagues et éliminations normales jusqu’au verdict du moteur.</x:v>
+      </x:c>
+      <x:c r="F142" s="51" t="str">
+        <x:v>Même protocole automatisé ; ce n’est pas une partie humaine ni une preuve d’équilibrage.</x:v>
+      </x:c>
+      <x:c r="G142" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H142" s="51" t="str">
+        <x:v>scripts/browserSceneServices.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="72" customHeight="1">
+      <x:c r="A143" s="52" t="str">
+        <x:v>SUITE-INFESTATION</x:v>
+      </x:c>
+      <x:c r="B143" s="51" t="str">
+        <x:v>Partie par entrées automatisées</x:v>
+      </x:c>
+      <x:c r="C143" s="51" t="str">
+        <x:v>Victoire à 3 600 frames</x:v>
+      </x:c>
+      <x:c r="D143" s="51" t="str">
+        <x:v>14, 15, 16 / HUB-04, HUB-05</x:v>
+      </x:c>
+      <x:c r="E143" s="51" t="str">
+        <x:v>Survie 60 secondes simulées ; briefing aligné sur la règle existante.</x:v>
+      </x:c>
+      <x:c r="F143" s="51" t="str">
+        <x:v>Horloge virtuelle ; ne mesure pas les performances réelles pendant 60 secondes.</x:v>
+      </x:c>
+      <x:c r="G143" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H143" s="51" t="str">
+        <x:v>scripts/browserSceneServices.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="72" customHeight="1">
+      <x:c r="A144" s="52" t="str">
+        <x:v>SUITE-HUNT</x:v>
+      </x:c>
+      <x:c r="B144" s="51" t="str">
+        <x:v>Partie par entrées automatisées</x:v>
+      </x:c>
+      <x:c r="C144" s="51" t="str">
+        <x:v>Victoire</x:v>
+      </x:c>
+      <x:c r="D144" s="51" t="str">
+        <x:v>15, 16 / HUB-04, HUB-05</x:v>
+      </x:c>
+      <x:c r="E144" s="51" t="str">
+        <x:v>Run Chasse : apparition et élimination du champion par tirs et compétence légaux.</x:v>
+      </x:c>
+      <x:c r="F144" s="51" t="str">
+        <x:v>Pas de fin forcée ; ne couvre pas chaque héros ni chaque arme.</x:v>
+      </x:c>
+      <x:c r="G144" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H144" s="51" t="str">
+        <x:v>scripts/browserSceneServices.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="72" customHeight="1">
+      <x:c r="A145" s="52" t="str">
+        <x:v>SUITE-LANGUES</x:v>
+      </x:c>
+      <x:c r="B145" s="51" t="str">
+        <x:v>Tests de présentation</x:v>
+      </x:c>
+      <x:c r="C145" s="51" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D145" s="51" t="str">
+        <x:v>14–19 / HUB-04, HUB-06</x:v>
+      </x:c>
+      <x:c r="E145" s="51" t="str">
+        <x:v>5 familles d’objectifs Course FR/EN ; 6 types ennemis Extinction ; noms d’armes ramassées.</x:v>
+      </x:c>
+      <x:c r="F145" s="51" t="str">
+        <x:v>Identifiants internes, IA, récompenses et progression inchangés ; autres textes de catalogue encore mixtes.</x:v>
+      </x:c>
+      <x:c r="G145" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H145" s="51" t="str">
+        <x:v>src/game/scenePresentation.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="72" customHeight="1">
+      <x:c r="A146" s="52" t="str">
+        <x:v>SUITE-UNIT</x:v>
+      </x:c>
+      <x:c r="B146" s="51" t="str">
+        <x:v>Tests unitaires locaux</x:v>
+      </x:c>
+      <x:c r="C146" s="51" t="str">
+        <x:v>81/81 réussis</x:v>
+      </x:c>
+      <x:c r="D146" s="51" t="str">
+        <x:v>Cité, Extinction, Course</x:v>
+      </x:c>
+      <x:c r="E146" s="51" t="str">
+        <x:v>node --test : présentation, entrées, temps, Cité, état du Hub, gameplay Fighter/Course.</x:v>
+      </x:c>
+      <x:c r="F146" s="51" t="str">
+        <x:v>Recoupement avec les autres suites : ne pas additionner comme tests tous distincts.</x:v>
+      </x:c>
+      <x:c r="G146" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H146" s="51" t="str">
+        <x:v>scripts/scenePresentation.test.mjs ; suites existantes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="72" customHeight="1">
+      <x:c r="A147" s="52" t="str">
+        <x:v>SUITE-UI</x:v>
+      </x:c>
+      <x:c r="B147" s="51" t="str">
+        <x:v>Tests unitaires locaux</x:v>
+      </x:c>
+      <x:c r="C147" s="51" t="str">
+        <x:v>68/68 réussis</x:v>
+      </x:c>
+      <x:c r="D147" s="51" t="str">
+        <x:v>Transversal</x:v>
+      </x:c>
+      <x:c r="E147" s="51" t="str">
+        <x:v>npm run test:ui-immersion</x:v>
+      </x:c>
+      <x:c r="F147" s="51" t="str">
+        <x:v>Contrats automatisés ; ne remplace pas la recette visuelle des 40 écrans.</x:v>
+      </x:c>
+      <x:c r="G147" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H147" s="51" t="str">
+        <x:v>package.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="72" customHeight="1">
+      <x:c r="A148" s="52" t="str">
+        <x:v>SUITE-LINT</x:v>
+      </x:c>
+      <x:c r="B148" s="51" t="str">
+        <x:v>Analyse statique locale</x:v>
+      </x:c>
+      <x:c r="C148" s="51" t="str">
+        <x:v>0 erreur / 0 avertissement</x:v>
+      </x:c>
+      <x:c r="D148" s="51" t="str">
+        <x:v>7 modules/tests</x:v>
+      </x:c>
+      <x:c r="E148" s="51" t="str">
+        <x:v>oxlint --max-warnings 0 sur les sept fichiers concernés.</x:v>
+      </x:c>
+      <x:c r="F148" s="51" t="str">
+        <x:v>Périmètre ciblé ; pas une certification de tout le dépôt.</x:v>
+      </x:c>
+      <x:c r="G148" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H148" s="51" t="str">
+        <x:v>source-manifest de la reprise</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="72" customHeight="1">
+      <x:c r="A149" s="52" t="str">
+        <x:v>SUITE-BUILD</x:v>
+      </x:c>
+      <x:c r="B149" s="51" t="str">
+        <x:v>Compilation locale</x:v>
+      </x:c>
+      <x:c r="C149" s="51" t="str">
+        <x:v>Réussie</x:v>
+      </x:c>
+      <x:c r="D149" s="51" t="str">
+        <x:v>Source snapshot</x:v>
+      </x:c>
+      <x:c r="E149" s="51" t="str">
+        <x:v>vite build sur les sources et médias disponibles.</x:v>
+      </x:c>
+      <x:c r="F149" s="51" t="str">
+        <x:v>Pas le prebuild complet ; avertissement de taille de bundle conservé.</x:v>
+      </x:c>
+      <x:c r="G149" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+      </x:c>
+      <x:c r="H149" s="51" t="str">
+        <x:v>journaux source-build.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="72" customHeight="1">
+      <x:c r="A150" s="52" t="str">
+        <x:v>SUITE-CI</x:v>
+      </x:c>
+      <x:c r="B150" s="51" t="str">
+        <x:v>Vérification distante</x:v>
+      </x:c>
+      <x:c r="C150" s="51" t="str">
+        <x:v>À confirmer dans Checks</x:v>
+      </x:c>
+      <x:c r="D150" s="51" t="str">
+        <x:v>Reprise du 26 octobre 2026</x:v>
+      </x:c>
+      <x:c r="E150" s="51" t="str">
+        <x:v>Suites permanentes Cité/Extinction et Course étendues ; reçu CI à consulter.</x:v>
+      </x:c>
+      <x:c r="F150" s="51" t="str">
+        <x:v>État à la préparation de ce fichier. Le reçu complète les résultats sans réécrire l’historique.</x:v>
+      </x:c>
+      <x:c r="G150" s="51" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/pull/9/checks</x:v>
+      </x:c>
+      <x:c r="H150" s="51" t="str">
+        <x:v>.github/workflows/city-extinction-ui.yml ; race-ui.yml</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12053,7 +12364,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7f13efc895044e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfb2a8faaba94659"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ec): publish verified workbook refresh and owner-resolved FPS checks
Integrate the exact nine blobs validated by run 40525781811: 127 targeted tests, 6 catalogue tests, 210518 compared production cells, both workbooks checked. Replace stale hardcoded Mirelle source assertion with owner binding regression coverage, retain runtime contract. Remove all ten temporary delivery/readback files. No gameplay asset completion or production certification claimed.
</commit_message>
<xml_diff>
--- a/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
+++ b/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Ra66e7982a0454dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="R42ab32bf09e24aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="R63fa9931639b4299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R70aac3a595cf4685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="R93fc1939b7244690"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Ra9fe647cab9e40d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Racce51ec46ff4893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="R4c1aec1f1d6e40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R937f9466b64d4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="Raf67dc8bf95f4636"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -655,8 +655,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H150" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:H150"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H162" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:H162"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Réf."/>
     <x:tableColumn id="2" name="Nature de preuve"/>
@@ -913,7 +913,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>Suivi continu de l’audit des 40 écrans — journal, services et parties Extinction du 26 octobre 2026.</x:v>
+        <x:v>Suivi continu des 40 écrans — reprise habitants Cité et cadrage FPS, 27 octobre 2026 ; PR nº 11.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1456,7 +1456,7 @@
     </x:row>
     <x:row r="40" ht="35" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>Sources : audit initial, ledgers, validation.json et comptes rendus de reprise Fighter, Course, Cité/Extinction.</x:v>
+        <x:v>Sources : audit initial et reçus historiques conservés ; nouvelle preuve : docs/extinction-city/residents-fps-ci-receipt-2026-10-27.json.</x:v>
       </x:c>
       <x:c r="B40" s="2"/>
       <x:c r="C40" s="2"/>
@@ -1468,7 +1468,7 @@
     </x:row>
     <x:row r="41" ht="35" customHeight="1">
       <x:c r="A41" s="7" t="str">
-        <x:v>26 octobre 2026 : composants réels, progression préparée et fins injectées ; matériel physique, compte cloud et recette complète restent ouverts.</x:v>
+        <x:v>27/10 : 12 approches de trois habitants ; 6 parcours de cadrage FPS. Possession préparée/horloge virtuelle ; pas de recette exhaustive, compte réel ou appareil physique.</x:v>
       </x:c>
       <x:c r="B41" s="2"/>
       <x:c r="C41" s="2"/>
@@ -4956,7 +4956,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2393ffe42bdb490e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83666955b4f14b5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5872,7 +5872,8 @@
 Position, orientation et quartier sont sauvegardés dans activityProgress.mosaicLocation toutes les cinq secondes, à la sortie et au pagehide. Retour sûr à l’Atrium si le quartier devient indisponible.
 Services connectés : Archives → Codex ; chambre des arcs → arcs ; relectures → journal ; récupération → équipe ; reliques → inventaire ; simulateur → Custom. La navigation mission conserve le contexte de l’univers malgré la remise à zéro des sous-vues.
 Suite du 26/10 : les habitants gardent leurs positions lors des réaffichages équivalents du parent. Le terminal annule le trajet et les entrées ; déplacement maintenu indépendant par touche/pointeur. Reprise après erreur sans téléporter l’Ancre ; cadrage de mini-carte borné au quartier.
-Suite suivante : Transmission ouvrable directement au HUD agrandi. Snapshot explicite avant chaque sortie de service, y compris missions et codex ; commandes relâchées et menu fermé. 36 transitions contrôlées sur quatre formats.</x:v>
+Suite suivante : Transmission ouvrable directement au HUD agrandi. Snapshot explicite avant chaque sortie de service, y compris missions et codex ; commandes relâchées et menu fermé. 36 transitions contrôlées sur quatre formats.
+27/10 — Répertoire complet des habitants possédés/visibles, recherche et pages de neuf ; groupes bornés à 17 plus Mirelle. Rejoindre marche vers l’identité ; détours autour des PNJ, suivi des habitants qui bougent, annulation au clavier/terminal.</x:v>
       </x:c>
       <x:c r="H20" s="21" t="str">
         <x:v>src/components/HubScreen.jsx
@@ -5882,7 +5883,8 @@
 src/game/immersiveHubState.js
 scripts/mosaicCityRuntime.test.mjs
 scripts/immersiveHubState.test.mjs
-src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx
+src/game/mosaicResidents.js ; src/game/mosaicCityRuntime.js ; scripts/mosaicResidentNavigation.test.mjs ; scripts/browserResidentViewmodels.py</x:v>
       </x:c>
       <x:c r="I20" s="21" t="str">
         <x:v>34 tests mosaicCityRuntime réussis, dont navigation de proximité, destinations autorisées, tutoriel, collisions et entrées clavier/tactiles.
@@ -5892,13 +5894,16 @@
 git diff --check : succès.
 26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
 Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677
-Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.</x:v>
+Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.
+Reprise CI : 121 tests ciblés et 68 UI, avec recoupements ; 12 approches sur trois identités dans quatre formats.</x:v>
       </x:c>
       <x:c r="J20" s="21" t="str">
-        <x:v>Destinations préparées : neuf accès représentatifs, quatre tailles ; pas tous les quartiers ni les écrans de destination réels. Validation artistique globale, appareil physique et cloud non effectués.</x:v>
+        <x:v>Destinations préparées : neuf accès représentatifs, quatre tailles ; pas tous les quartiers ni les écrans de destination réels. Validation artistique globale, appareil physique et cloud non effectués.
+Non exhaustif : trois habitants parcourus, possession préparée, pas tous les quartiers/services ni matériel réel.</x:v>
       </x:c>
       <x:c r="K20" s="21" t="str">
-        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json
+https://github.com/darknigthmare/multiverse-breach/blob/dc95aec15309fb2f9a23e36971b30db46197f9a6/docs/extinction-city/residents-fps-ci-receipt-2026-10-27.json</x:v>
       </x:c>
       <x:c r="L20" s="27" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -5939,13 +5944,15 @@
 Partie FPS dans une scène couvrant le viewport, avec objectif, PV/armure/munitions et commandes superposés aux bords. Radar, réticule, arme et simulation sont conservés.
 Suppression du doublon visuel des mêmes statistiques dans le canevas, puisque toutes restent présentes dans un HUD DOM lisible et accessible.
 Suite du 26/10 : une touche relâchée ne coupe plus un autre contrôle maintenu. Visée par pointeur propriétaire et seuil cumulé de glissement ; commandes tactiles capturées. Directive · Commandes suspend la simulation. HUD compact et contrôles adaptés au paysage court. Panne de rendu récupérable sans victoire.
-Suite suivante : objectif Infestation précise les 60 secondes existantes. Six noms ennemis et les armes ramassées suivent la langue d’interface, sans modifier les types internes. Les quatre variantes atteignent leur victoire par les entrées normales.</x:v>
+Suite suivante : objectif Infestation précise les 60 secondes existantes. Six noms ennemis et les armes ramassées suivent la langue d’interface, sans modifier les types internes. Les quatre variantes atteignent leur victoire par les entrées normales.
+27/10 — Mains FPS et effet visuel gardent leurs proportions ; rognage dans la cellule déclarée, recharge Mirelle ligne 6/marges 40 et 6. Replis neutres et identités préservés.</x:v>
       </x:c>
       <x:c r="H21" s="22" t="str">
         <x:v>src/components/HubScreen.jsx
 src/components/HubImmersion.css
 src/components/useSceneViewport.js
-src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx</x:v>
+src/game/sceneInputs.js ; src/components/SceneHoldButton.jsx ; scripts/browserCityExtinction.py ; scripts/fixtures/cityExtinctionHarness.jsx
+src/game/extinctionContent.js ; scripts/extinctionViewmodelContract.mjs ; scripts/browserResidentViewmodels.py</x:v>
       </x:c>
       <x:c r="I21" s="22" t="str">
         <x:v>extinctionTiming : simulation réelle, dégâts, déplacements et recharge identiques à 30/60/120/144 Hz ; pause et visibilité sans rattrapage.
@@ -5954,13 +5961,16 @@
 git diff --check : succès.
 26/10 : 64 tests scènes/entrées/temps/Hub et 68 tests UI existants réussis localement ; suites se recoupant. Réexécution avec médias du dépôt dans le workflow dédié.
 Exécution distante 40279377677 : 64/64 + 68/68, lint 0/0, compilation source et 10/10 parcours Chromium avec médias réussis. https://github.com/darknigthmare/multiverse-breach/actions/runs/40279377677
-Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.</x:v>
+Suite suivante : 81 tests ciblés / 68 UI ; parcours décrits dans le reçu de reprise.
+Six scénarios de cadrage/tir/recharge et six anciens scénarios de sélection réussis. Contrat de progression exécutable avec tests négatifs.</x:v>
       </x:c>
       <x:c r="J21" s="22" t="str">
-        <x:v>Quatre victoires automatisées avec horloge virtuelle et un profil préparé. Pas de test humain, d’équilibrage ou de tous les héros/armes. Silhouettes génériques inchangées ; autres libellés à relire.</x:v>
+        <x:v>Quatre victoires automatisées avec horloge virtuelle et un profil préparé. Pas de test humain, d’équilibrage ou de tous les héros/armes. Silhouettes génériques inchangées ; autres libellés à relire.
+Trois raccordements artistiques seulement partiels ; pas de nouvelles mains, animations de toutes tenues, projectiles physiques ou bestiaire.</x:v>
       </x:c>
       <x:c r="K21" s="22" t="str">
-        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/docs/ui-immersion/scene-completion-2026-10-26.json
+https://github.com/darknigthmare/multiverse-breach/blob/dc95aec15309fb2f9a23e36971b30db46197f9a6/docs/extinction-city/residents-fps-ci-receipt-2026-10-27.json</x:v>
       </x:c>
       <x:c r="L21" s="26" t="str">
         <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/blob/codex/immersive-ui-audit-2026-10-25/src/components/HubScreen.jsx","Code de la branche"),"Code de la branche")</x:f>
@@ -7379,7 +7389,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc922c48618ae473c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6653d5043ba47e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8661,7 +8671,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd7837f16ee743d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6debbdeb143941cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12334,6 +12344,318 @@
       </x:c>
       <x:c r="H150" s="51" t="str">
         <x:v>.github/workflows/city-extinction-ui.yml ; race-ui.yml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="150" customHeight="1">
+      <x:c r="A151" s="50" t="str">
+        <x:v>EC27-BASE</x:v>
+      </x:c>
+      <x:c r="B151" s="50" t="str">
+        <x:v>Publication source</x:v>
+      </x:c>
+      <x:c r="C151" s="50" t="str">
+        <x:v>Publié</x:v>
+      </x:c>
+      <x:c r="D151" s="50" t="str">
+        <x:v>Cité / Extinction</x:v>
+      </x:c>
+      <x:c r="E151" s="50" t="str">
+        <x:v>Source dc95aec15309fb2f9a23e36971b30db46197f9a6 ; PR nº 11 après fusion de nº 9.</x:v>
+      </x:c>
+      <x:c r="F151" s="50" t="str">
+        <x:v>Aucune fusion ni promotion de production ; autres PR inchangées.</x:v>
+      </x:c>
+      <x:c r="G151" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/blob/dc95aec15309fb2f9a23e36971b30db46197f9a6/docs/extinction-city/residents-fps-ci-receipt-2026-10-27.json</x:v>
+      </x:c>
+      <x:c r="H151" s="50" t="str">
+        <x:v>GitHub / base master 1460d0e</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="150" customHeight="1">
+      <x:c r="A152" s="50" t="str">
+        <x:v>EC27-UNIT</x:v>
+      </x:c>
+      <x:c r="B152" s="50" t="str">
+        <x:v>Tests unitaires CI et locaux</x:v>
+      </x:c>
+      <x:c r="C152" s="50" t="str">
+        <x:v>121/121 réussis</x:v>
+      </x:c>
+      <x:c r="D152" s="50" t="str">
+        <x:v>Commandes, temps, Cité, FPS, progression</x:v>
+      </x:c>
+      <x:c r="E152" s="50" t="str">
+        <x:v>Suite ciblée ; six nouveaux tests des trajets autour des PNJ, cible mouvante et annulation.</x:v>
+      </x:c>
+      <x:c r="F152" s="50" t="str">
+        <x:v>Ces suites se recoupent avec les tests UI ; ne pas additionner comme tests uniques.</x:v>
+      </x:c>
+      <x:c r="G152" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H152" s="50" t="str">
+        <x:v>unit.log / scripts/mosaicResidentNavigation.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="150" customHeight="1">
+      <x:c r="A153" s="50" t="str">
+        <x:v>EC27-UI</x:v>
+      </x:c>
+      <x:c r="B153" s="50" t="str">
+        <x:v>Tests unitaires CI</x:v>
+      </x:c>
+      <x:c r="C153" s="50" t="str">
+        <x:v>68/68 réussis</x:v>
+      </x:c>
+      <x:c r="D153" s="50" t="str">
+        <x:v>Interface immersive</x:v>
+      </x:c>
+      <x:c r="E153" s="50" t="str">
+        <x:v>npm run test:ui-immersion</x:v>
+      </x:c>
+      <x:c r="F153" s="50" t="str">
+        <x:v>Contrats et rendu préparé ; pas une recette visuelle exhaustive des 40 écrans.</x:v>
+      </x:c>
+      <x:c r="G153" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H153" s="50" t="str">
+        <x:v>ui.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="150" customHeight="1">
+      <x:c r="A154" s="50" t="str">
+        <x:v>EC27-CITY-P</x:v>
+      </x:c>
+      <x:c r="B154" s="50" t="str">
+        <x:v>Navigateur Chromium</x:v>
+      </x:c>
+      <x:c r="C154" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D154" s="50" t="str">
+        <x:v>Cité / 390×844 EN</x:v>
+      </x:c>
+      <x:c r="E154" s="50" t="str">
+        <x:v>Rejoindre trois habitants depuis le répertoire, dont deux non-combattants ; dialogue accessible.</x:v>
+      </x:c>
+      <x:c r="F154" s="50" t="str">
+        <x:v>Possession préparée et horloge virtuelle. Pas de téléportation ; seulement ces trois identités.</x:v>
+      </x:c>
+      <x:c r="G154" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H154" s="50" t="str">
+        <x:v>city-residents-390x844-en</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="150" customHeight="1">
+      <x:c r="A155" s="50" t="str">
+        <x:v>EC27-CITY-D</x:v>
+      </x:c>
+      <x:c r="B155" s="50" t="str">
+        <x:v>Navigateur Chromium</x:v>
+      </x:c>
+      <x:c r="C155" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D155" s="50" t="str">
+        <x:v>Cité / 1280×900 FR</x:v>
+      </x:c>
+      <x:c r="E155" s="50" t="str">
+        <x:v>Rejoindre trois habitants, dont Bastion malgré un PNJ interposé ; réaffichage sans perte de position.</x:v>
+      </x:c>
+      <x:c r="F155" s="50" t="str">
+        <x:v>Possession préparée ; pas tous les quartiers ni tous les services.</x:v>
+      </x:c>
+      <x:c r="G155" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H155" s="50" t="str">
+        <x:v>city-residents-1280x900-fr</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="150" customHeight="1">
+      <x:c r="A156" s="50" t="str">
+        <x:v>EC27-CITY-L</x:v>
+      </x:c>
+      <x:c r="B156" s="50" t="str">
+        <x:v>Navigateur Chromium</x:v>
+      </x:c>
+      <x:c r="C156" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D156" s="50" t="str">
+        <x:v>Cité / 844×390 FR</x:v>
+      </x:c>
+      <x:c r="E156" s="50" t="str">
+        <x:v>Recherche, répertoire, approche et dialogue des trois identités.</x:v>
+      </x:c>
+      <x:c r="F156" s="50" t="str">
+        <x:v>Fenêtre navigateur en paysage ; pas un téléphone physique.</x:v>
+      </x:c>
+      <x:c r="G156" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H156" s="50" t="str">
+        <x:v>city-residents-844x390-fr</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="150" customHeight="1">
+      <x:c r="A157" s="50" t="str">
+        <x:v>EC27-CITY-U</x:v>
+      </x:c>
+      <x:c r="B157" s="50" t="str">
+        <x:v>Navigateur Chromium</x:v>
+      </x:c>
+      <x:c r="C157" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D157" s="50" t="str">
+        <x:v>Cité / 2560×1080 EN</x:v>
+      </x:c>
+      <x:c r="E157" s="50" t="str">
+        <x:v>Recherche, répertoire, approche et dialogue des trois identités.</x:v>
+      </x:c>
+      <x:c r="F157" s="50" t="str">
+        <x:v>Trois habitants, pas 1 911 personnages parcourus ; les autres restent indexés.</x:v>
+      </x:c>
+      <x:c r="G157" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H157" s="50" t="str">
+        <x:v>city-residents-2560x1080-en</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="150" customHeight="1">
+      <x:c r="A158" s="50" t="str">
+        <x:v>EC27-FPS</x:v>
+      </x:c>
+      <x:c r="B158" s="50" t="str">
+        <x:v>Appels de dessin + commandes natives</x:v>
+      </x:c>
+      <x:c r="C158" s="50" t="str">
+        <x:v>6/6 réussis</x:v>
+      </x:c>
+      <x:c r="D158" s="50" t="str">
+        <x:v>Mirelle ×4 ; Arthur et Serj ×1</x:v>
+      </x:c>
+      <x:c r="E158" s="50" t="str">
+        <x:v>Tir consomme une munition ; recharge après retour au repos. Cellules source et proportions vérifiées.</x:v>
+      </x:c>
+      <x:c r="F158" s="50" t="str">
+        <x:v>Pas de nouveaux PNG, ni projectile physique, ni certification artistique ou de toutes les tenues.</x:v>
+      </x:c>
+      <x:c r="G158" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H158" s="50" t="str">
+        <x:v>browser/results.json / scripts/browserResidentViewmodels.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="150" customHeight="1">
+      <x:c r="A159" s="50" t="str">
+        <x:v>EC27-ROSTER</x:v>
+      </x:c>
+      <x:c r="B159" s="50" t="str">
+        <x:v>Régressions navigateur existantes</x:v>
+      </x:c>
+      <x:c r="C159" s="50" t="str">
+        <x:v>6/6 réussis</x:v>
+      </x:c>
+      <x:c r="D159" s="50" t="str">
+        <x:v>Sélection et identité FPS</x:v>
+      </x:c>
+      <x:c r="E159" s="50" t="str">
+        <x:v>Mains attendues décodées ; profil sans mains, combattant en fin de liste et liste vide.</x:v>
+      </x:c>
+      <x:c r="F159" s="50" t="str">
+        <x:v>Décors secondaires Arthur/Serj et portrait de fin de liste hors checkout : chargement non certifié.</x:v>
+      </x:c>
+      <x:c r="G159" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H159" s="50" t="str">
+        <x:v>existing/results.json / scripts/browserExtinctionCatalog.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="150" customHeight="1">
+      <x:c r="A160" s="50" t="str">
+        <x:v>EC27-LINT</x:v>
+      </x:c>
+      <x:c r="B160" s="50" t="str">
+        <x:v>Analyse statique CI</x:v>
+      </x:c>
+      <x:c r="C160" s="50" t="str">
+        <x:v>0 erreur / 0 avertissement</x:v>
+      </x:c>
+      <x:c r="D160" s="50" t="str">
+        <x:v>8 modules/tests</x:v>
+      </x:c>
+      <x:c r="E160" s="50" t="str">
+        <x:v>oxlint --max-warnings 0</x:v>
+      </x:c>
+      <x:c r="F160" s="50" t="str">
+        <x:v>Périmètre ciblé, pas audit de toutes les dépendances.</x:v>
+      </x:c>
+      <x:c r="G160" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H160" s="50" t="str">
+        <x:v>lint.log</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="150" customHeight="1">
+      <x:c r="A161" s="50" t="str">
+        <x:v>EC27-BUILD</x:v>
+      </x:c>
+      <x:c r="B161" s="50" t="str">
+        <x:v>Compilation Vite source CI</x:v>
+      </x:c>
+      <x:c r="C161" s="50" t="str">
+        <x:v>Réussie</x:v>
+      </x:c>
+      <x:c r="D161" s="50" t="str">
+        <x:v>Snapshot partiel</x:v>
+      </x:c>
+      <x:c r="E161" s="50" t="str">
+        <x:v>Vite build ; contrat exécutable des mains remplace les anciennes recherches de texte.</x:v>
+      </x:c>
+      <x:c r="F161" s="50" t="str">
+        <x:v>Ne vaut pas build complet. Les checks du dernier commit sont distincts.</x:v>
+      </x:c>
+      <x:c r="G161" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40508601682</x:v>
+      </x:c>
+      <x:c r="H161" s="50" t="str">
+        <x:v>source-build.log / scripts/extinctionViewmodelContract.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="150" customHeight="1">
+      <x:c r="A162" s="50" t="str">
+        <x:v>EC27-OPEN</x:v>
+      </x:c>
+      <x:c r="B162" s="50" t="str">
+        <x:v>Reste à réaliser</x:v>
+      </x:c>
+      <x:c r="C162" s="50" t="str">
+        <x:v>Ouvert</x:v>
+      </x:c>
+      <x:c r="D162" s="50" t="str">
+        <x:v>Univers, personnages, ennemis, boss, zones et props</x:v>
+      </x:c>
+      <x:c r="E162" s="50" t="str">
+        <x:v>Voir le second Excel actualisé, ses 23 lignes de recette et ses 17 732 lignes de catalogue.</x:v>
+      </x:c>
+      <x:c r="F162" s="50" t="str">
+        <x:v>Bot Infestation intermittent ; assets spécifiques, actions individuelles, services réels, matériel et cloud restent ouverts.</x:v>
+      </x:c>
+      <x:c r="G162" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/pull/11/checks</x:v>
+      </x:c>
+      <x:c r="H162" s="50" t="str">
+        <x:v>docs/excel/Multiverse_Breach_Extinction_Cite_Production.xlsx</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12364,7 +12686,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfb2a8faaba94659"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1c3b11876894089"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(ec): publish verified Nexus protocols workbooks and preserve audit history
Integrate exact exports verified by run 40725181635: 17741 production rows, 210557 compared cells, 170 UI checks with all 156 historical rows preserved, formula KPIs 7/28/1587 and no cached formula errors. Pin the permanent workbook workflow to the new receipt. Remove thirteen temporary transport files. Existing source was verified by run 40719252474; full production checks remain separate.
</commit_message>
<xml_diff>
--- a/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
+++ b/docs/excel/Multiverse_Breach_UI_Immersion.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="Ra9fe647cab9e40d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Racce51ec46ff4893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="R4c1aec1f1d6e40cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="R937f9466b64d4c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="Raf67dc8bf95f4636"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R8abffb8ee9f646ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40 écrans" sheetId="2" r:id="Rf5c2ec02092e4ded"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="3" r:id="Rcf43bcbb9fb04f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conservation" sheetId="4" r:id="Re8397416ac8943cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vérifications" sheetId="5" r:id="R1440af82953e4413"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -655,8 +655,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H162" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:H162"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ImmersionVerification" displayName="ImmersionVerification" ref="A6:H176" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:H176"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Réf."/>
     <x:tableColumn id="2" name="Nature de preuve"/>
@@ -913,7 +913,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>Suivi continu des 40 écrans — reprise habitants Cité et cadrage FPS, 27 octobre 2026 ; PR nº 11.</x:v>
+        <x:v>Reprise du 28 octobre 2026 — sept kits FPS Nexus et vitrines d’archives ; suite de la PR nº 11 fusionnée.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1159,7 +1159,7 @@
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="46" t="str">
-        <x:v>Journal Cité ouvrable au HUD agrandi ; 36 transitions de services ; quatre variantes Extinction terminées par entrées automatisées.</x:v>
+        <x:v>7 kits Nexus : 28 actions jouables. Vitrines consultables ; aucune attribution d’objet. Art et autres univers toujours partiels.</x:v>
       </x:c>
       <x:c r="B16" s="2"/>
       <x:c r="C16" s="2"/>
@@ -1267,7 +1267,7 @@
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="46" t="str">
-        <x:v>Suite : 81 tests ciblés, 68 tests UI (recoupements), quatre parcours Cité et quatre runs Extinction ; état distant dans Checks.</x:v>
+        <x:v>155 tests ciblés, 68 UI, 7 catalogue ; 14 nouveaux scénarios navigateur préparés. Les suites se recoupent.</x:v>
       </x:c>
       <x:c r="B25" s="2"/>
       <x:c r="C25" s="2"/>
@@ -1365,7 +1365,7 @@
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="47" t="str">
-        <x:v>codex/immersive-ui-audit-2026-10-25</x:v>
+        <x:v>codex/ec-backlog-2026-10-28</x:v>
       </x:c>
       <x:c r="D33" s="2"/>
       <x:c r="E33" s="2"/>
@@ -1379,7 +1379,7 @@
       </x:c>
       <x:c r="B34" s="2"/>
       <x:c r="C34" s="47" t="str">
-        <x:v>b8b2c326da45ce11ed8bd8868fca0bf266dfd31a</x:v>
+        <x:v>fed79e8fdbcc811616bd0ec6f3a73b9656b5d8b9</x:v>
       </x:c>
       <x:c r="D34" s="2"/>
       <x:c r="E34" s="2"/>
@@ -1393,7 +1393,7 @@
       </x:c>
       <x:c r="B35" s="2"/>
       <x:c r="C35" s="47" t="str">
-        <x:v>Base d915220 / snapshot c7ce3caf ; preuves : scene-completion-2026-10-26.json et reçu CI lié dans la PR.</x:v>
+        <x:v>849ae4eea0b761df0b518a815132a458ecfca2c7 ; code exact validé dans le run 40719252474.</x:v>
       </x:c>
       <x:c r="D35" s="2"/>
       <x:c r="E35" s="2"/>
@@ -1403,12 +1403,11 @@
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
       <x:c r="A36" s="2" t="str">
-        <x:v>Pull request</x:v>
+        <x:v>Continuation</x:v>
       </x:c>
       <x:c r="B36" s="2"/>
       <x:c r="C36" s="47" t="str">
-        <x:f>IFERROR(HYPERLINK("https://github.com/darknigthmare/multiverse-breach/pull/9","Ouvrir la pull request"),"Ouvrir la pull request")</x:f>
-        <x:v>Ouvrir la pull request</x:v>
+        <x:v>https://github.com/darknigthmare/multiverse-breach/tree/codex/ec-backlog-2026-10-28</x:v>
       </x:c>
       <x:c r="D36" s="2"/>
       <x:c r="E36" s="2"/>
@@ -1436,7 +1435,7 @@
       </x:c>
       <x:c r="B38" s="2"/>
       <x:c r="C38" s="47" t="str">
-        <x:v>Actualisation artifact_tool ; historique conservé ; 144 vérifications. Aucun écran déclaré entièrement validé par cette passe.</x:v>
+        <x:v>Actualisation artifact_tool ; 170 vérifications dont 156 historiques conservées. Aucun écran entièrement certifié par cette passe.</x:v>
       </x:c>
       <x:c r="D38" s="2"/>
       <x:c r="E38" s="2"/>
@@ -1456,7 +1455,7 @@
     </x:row>
     <x:row r="40" ht="35" customHeight="1">
       <x:c r="A40" s="7" t="str">
-        <x:v>Sources : audit initial et reçus historiques conservés ; nouvelle preuve : docs/extinction-city/residents-fps-ci-receipt-2026-10-27.json.</x:v>
+        <x:v>Sources historiques conservées ; continuation : docs/extinction-city/protocols-2026-10-28.json.</x:v>
       </x:c>
       <x:c r="B40" s="2"/>
       <x:c r="C40" s="2"/>
@@ -4956,7 +4955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83666955b4f14b5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4ad79b7e93248b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7389,7 +7388,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6653d5043ba47e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R723f33ac3898453e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8671,7 +8670,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6debbdeb143941cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55444ea0d4424310"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12656,6 +12655,370 @@
       </x:c>
       <x:c r="H162" s="50" t="str">
         <x:v>docs/excel/Multiverse_Breach_Extinction_Cite_Production.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="102" customHeight="1">
+      <x:c r="A163" s="50" t="str">
+        <x:v>EC28-KITS</x:v>
+      </x:c>
+      <x:c r="B163" s="50" t="str">
+        <x:v>Adaptation source exécutée</x:v>
+      </x:c>
+      <x:c r="C163" s="50" t="str">
+        <x:v>28 actions / 7 identités</x:v>
+      </x:c>
+      <x:c r="D163" s="50" t="str">
+        <x:v>Ancre, Mirelle, Bastion, Nova, Marrow, Sable, Loom</x:v>
+      </x:c>
+      <x:c r="E163" s="50" t="str">
+        <x:v>Tir/attaque, secondaire, défense, ultime ; noms et types source conservés.</x:v>
+      </x:c>
+      <x:c r="F163" s="50" t="str">
+        <x:v>Compression FPS propre au jeu. Aucune certification canonique ou art individuel complet.</x:v>
+      </x:c>
+      <x:c r="G163" s="50" t="str">
+        <x:v>src/game/extinctionSignatures.js</x:v>
+      </x:c>
+      <x:c r="H163" s="50" t="str">
+        <x:v>scripts/extinctionSignatures.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="102" customHeight="1">
+      <x:c r="A164" s="50" t="str">
+        <x:v>EC28-UNIT</x:v>
+      </x:c>
+      <x:c r="B164" s="50" t="str">
+        <x:v>Tests automatiques locaux</x:v>
+      </x:c>
+      <x:c r="C164" s="50" t="str">
+        <x:v>155/155 réussis</x:v>
+      </x:c>
+      <x:c r="D164" s="50" t="str">
+        <x:v>Scènes, horloge, entrées, cadrage et nouveaux protocoles</x:v>
+      </x:c>
+      <x:c r="E164" s="50" t="str">
+        <x:v>node --test : suite ciblée finale ; aucun test ignoré.</x:v>
+      </x:c>
+      <x:c r="F164" s="50" t="str">
+        <x:v>Recoupement avec UI et catalogue ; ne pas additionner comme tests uniques.</x:v>
+      </x:c>
+      <x:c r="G164" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+      <x:c r="H164" s="50" t="str">
+        <x:v>scripts/extinctionSignatures.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="102" customHeight="1">
+      <x:c r="A165" s="50" t="str">
+        <x:v>EC28-UI</x:v>
+      </x:c>
+      <x:c r="B165" s="50" t="str">
+        <x:v>Tests d’interface locaux</x:v>
+      </x:c>
+      <x:c r="C165" s="50" t="str">
+        <x:v>68/68 réussis</x:v>
+      </x:c>
+      <x:c r="D165" s="50" t="str">
+        <x:v>Conservation de l’interface immersive</x:v>
+      </x:c>
+      <x:c r="E165" s="50" t="str">
+        <x:v>npm run test:ui-immersion</x:v>
+      </x:c>
+      <x:c r="F165" s="50" t="str">
+        <x:v>Ne remplace pas une revue humaine des 40 écrans.</x:v>
+      </x:c>
+      <x:c r="G165" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+      <x:c r="H165" s="50" t="str">
+        <x:v>package.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="102" customHeight="1">
+      <x:c r="A166" s="50" t="str">
+        <x:v>EC28-CATALOG</x:v>
+      </x:c>
+      <x:c r="B166" s="50" t="str">
+        <x:v>Contrats du catalogue</x:v>
+      </x:c>
+      <x:c r="C166" s="50" t="str">
+        <x:v>7/7 réussis</x:v>
+      </x:c>
+      <x:c r="D166" s="50" t="str">
+        <x:v>7 kits et 1 587 fiches de reliques</x:v>
+      </x:c>
+      <x:c r="E166" s="50" t="str">
+        <x:v>Catalogue exact ; autres kits non déclarés terminés.</x:v>
+      </x:c>
+      <x:c r="F166" s="50" t="str">
+        <x:v>Sources projet uniquement, pas validation externe des franchises.</x:v>
+      </x:c>
+      <x:c r="G166" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+      <x:c r="H166" s="50" t="str">
+        <x:v>scripts/extinctionCityCatalog.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="102" customHeight="1">
+      <x:c r="A167" s="50" t="str">
+        <x:v>EC28-PROJECTILES</x:v>
+      </x:c>
+      <x:c r="B167" s="50" t="str">
+        <x:v>Tests de simulation</x:v>
+      </x:c>
+      <x:c r="C167" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D167" s="50" t="str">
+        <x:v>Mirelle / Sable : projectile, roquette, mine</x:v>
+      </x:c>
+      <x:c r="E167" s="50" t="str">
+        <x:v>Impact différé, segment balayé, cible proche d’abord, TTL, pause, fin et propriétaire.</x:v>
+      </x:c>
+      <x:c r="F167" s="50" t="str">
+        <x:v>Rendu de secours procédural ; ni nouveaux PNG ni moteur balistique réaliste.</x:v>
+      </x:c>
+      <x:c r="G167" s="50" t="str">
+        <x:v>src/game/extinctionSignatures.js</x:v>
+      </x:c>
+      <x:c r="H167" s="50" t="str">
+        <x:v>scripts/extinctionSignatures.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="102" customHeight="1">
+      <x:c r="A168" s="50" t="str">
+        <x:v>EC28-SHIELD</x:v>
+      </x:c>
+      <x:c r="B168" s="50" t="str">
+        <x:v>Contrat de dégâts</x:v>
+      </x:c>
+      <x:c r="C168" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D168" s="50" t="str">
+        <x:v>Champion protégé et sources secondaires</x:v>
+      </x:c>
+      <x:c r="E168" s="50" t="str">
+        <x:v>Dégâts partagés entre protocoles, tourelle de rôle et ultime ramassé ; drones protecteurs respectés.</x:v>
+      </x:c>
+      <x:c r="F168" s="50" t="str">
+        <x:v>Pas une validation de tous les boss individuels du catalogue.</x:v>
+      </x:c>
+      <x:c r="G168" s="50" t="str">
+        <x:v>src/game/extinctionSignatures.js</x:v>
+      </x:c>
+      <x:c r="H168" s="50" t="str">
+        <x:v>scripts/extinctionSignatures.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="102" customHeight="1">
+      <x:c r="A169" s="50" t="str">
+        <x:v>EC28-BROWSER-FPS</x:v>
+      </x:c>
+      <x:c r="B169" s="50" t="str">
+        <x:v>Navigateur local, bundle en mémoire</x:v>
+      </x:c>
+      <x:c r="C169" s="50" t="str">
+        <x:v>10/10 réussis</x:v>
+      </x:c>
+      <x:c r="D169" s="50" t="str">
+        <x:v>7 identités Nexus ; 4 formats, FR/EN</x:v>
+      </x:c>
+      <x:c r="E169" s="50" t="str">
+        <x:v>Entrées Space puis F/C/X : charge gagnée par 13 attaques ; pause et abandon.</x:v>
+      </x:c>
+      <x:c r="F169" s="50" t="str">
+        <x:v>Cibles préparées et horloge virtuelle ; pas de victoire/récompense injectée. Pas un appareil physique.</x:v>
+      </x:c>
+      <x:c r="G169" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+      <x:c r="H169" s="50" t="str">
+        <x:v>scripts/browserExtinctionProtocols.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="102" customHeight="1">
+      <x:c r="A170" s="50" t="str">
+        <x:v>EC28-BROWSER-CITY</x:v>
+      </x:c>
+      <x:c r="B170" s="50" t="str">
+        <x:v>Navigateur local, bundle en mémoire</x:v>
+      </x:c>
+      <x:c r="C170" s="50" t="str">
+        <x:v>4/4 réussis</x:v>
+      </x:c>
+      <x:c r="D170" s="50" t="str">
+        <x:v>Vitrine Nexus : 390×844, 844×390, 1280×900, 2560×1080</x:v>
+      </x:c>
+      <x:c r="E170" s="50" t="str">
+        <x:v>Recherche, lecture, trajet natif, ouverture de fiche, pause et fermeture.</x:v>
+      </x:c>
+      <x:c r="F170" s="50" t="str">
+        <x:v>Une vitrine Nexus dans 4 formats, pas 525 quartiers parcourus ; aucune relique accordée.</x:v>
+      </x:c>
+      <x:c r="G170" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+      <x:c r="H170" s="50" t="str">
+        <x:v>scripts/browserExtinctionProtocols.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="102" customHeight="1">
+      <x:c r="A171" s="50" t="str">
+        <x:v>EC28-CITY-DATA</x:v>
+      </x:c>
+      <x:c r="B171" s="50" t="str">
+        <x:v>Contrat de conservation</x:v>
+      </x:c>
+      <x:c r="C171" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D171" s="50" t="str">
+        <x:v>1 587 fiches de reliques du catalogue</x:v>
+      </x:c>
+      <x:c r="E171" s="50" t="str">
+        <x:v>Filtre d’univers exact, possession/base+améliorée, désactivés, pagination ; consultation seule.</x:v>
+      </x:c>
+      <x:c r="F171" s="50" t="str">
+        <x:v>Les présentoirs communs ne sont pas 1 587 accessoires graphiques canoniques.</x:v>
+      </x:c>
+      <x:c r="G171" s="50" t="str">
+        <x:v>src/game/mosaicExhibits.js</x:v>
+      </x:c>
+      <x:c r="H171" s="50" t="str">
+        <x:v>scripts/mosaicExhibits.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="102" customHeight="1">
+      <x:c r="A172" s="50" t="str">
+        <x:v>EC28-ART-OWNER</x:v>
+      </x:c>
+      <x:c r="B172" s="50" t="str">
+        <x:v>Contrat de rendu</x:v>
+      </x:c>
+      <x:c r="C172" s="50" t="str">
+        <x:v>Réussi</x:v>
+      </x:c>
+      <x:c r="D172" s="50" t="str">
+        <x:v>Projectile Mirelle / repli neutre</x:v>
+      </x:c>
+      <x:c r="E172" s="50" t="str">
+        <x:v>Image existante seulement si propriétaire conforme et image chargée ; proportions conservées.</x:v>
+      </x:c>
+      <x:c r="F172" s="50" t="str">
+        <x:v>Trois planches FPS personnelles toujours seulement partiellement raccordées.</x:v>
+      </x:c>
+      <x:c r="G172" s="50" t="str">
+        <x:v>src/game/extinctionSignatures.js</x:v>
+      </x:c>
+      <x:c r="H172" s="50" t="str">
+        <x:v>scripts/extinctionSignatures.test.mjs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="102" customHeight="1">
+      <x:c r="A173" s="50" t="str">
+        <x:v>EC28-BUILD</x:v>
+      </x:c>
+      <x:c r="B173" s="50" t="str">
+        <x:v>Compilation locale des sources</x:v>
+      </x:c>
+      <x:c r="C173" s="50" t="str">
+        <x:v>Réussie</x:v>
+      </x:c>
+      <x:c r="D173" s="50" t="str">
+        <x:v>Copie source partielle</x:v>
+      </x:c>
+      <x:c r="E173" s="50" t="str">
+        <x:v>Vite build et lint ciblé sans erreur.</x:v>
+      </x:c>
+      <x:c r="F173" s="50" t="str">
+        <x:v>Prébuild complet avec tous les médias et checks du commit final à lire séparément.</x:v>
+      </x:c>
+      <x:c r="G173" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+      <x:c r="H173" s="50" t="str">
+        <x:v>vite.config.js</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="102" customHeight="1">
+      <x:c r="A174" s="50" t="str">
+        <x:v>EC28-OPEN</x:v>
+      </x:c>
+      <x:c r="B174" s="50" t="str">
+        <x:v>Reste à réaliser</x:v>
+      </x:c>
+      <x:c r="C174" s="50" t="str">
+        <x:v>Ouvert</x:v>
+      </x:c>
+      <x:c r="D174" s="50" t="str">
+        <x:v>Autres kits, art, ennemis, boss, décors, cloud et matériel</x:v>
+      </x:c>
+      <x:c r="E174" s="50" t="str">
+        <x:v>Production et recette restant ouvertes dans le second classeur.</x:v>
+      </x:c>
+      <x:c r="F174" s="50" t="str">
+        <x:v>Aucune suppression de contenu, aucun déblocage ou achat, aucun merge ou déploiement de production.</x:v>
+      </x:c>
+      <x:c r="G174" s="50" t="str">
+        <x:v>docs/excel/Multiverse_Breach_Extinction_Cite_Production.xlsx</x:v>
+      </x:c>
+      <x:c r="H174" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="102" customHeight="1">
+      <x:c r="A175" s="50" t="str">
+        <x:v>EC28-CI</x:v>
+      </x:c>
+      <x:c r="B175" s="50" t="str">
+        <x:v>Validation GitHub sur sources exactes</x:v>
+      </x:c>
+      <x:c r="C175" s="50" t="str">
+        <x:v>Réussie</x:v>
+      </x:c>
+      <x:c r="D175" s="50" t="str">
+        <x:v>13 fichiers code/tests ; source 849ae4e</x:v>
+      </x:c>
+      <x:c r="E175" s="50" t="str">
+        <x:v>155 ciblés, 68 UI, 7 catalogue, lint 7 fichiers, compilation source.</x:v>
+      </x:c>
+      <x:c r="F175" s="50" t="str">
+        <x:v>Fusion de test/commit final et prébuild production distincts ; suites se recoupent.</x:v>
+      </x:c>
+      <x:c r="G175" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40719252474</x:v>
+      </x:c>
+      <x:c r="H175" s="50" t="str">
+        <x:v>docs/extinction-city/protocols-2026-10-28.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="102" customHeight="1">
+      <x:c r="A176" s="50" t="str">
+        <x:v>EC28-CI-BROWSER</x:v>
+      </x:c>
+      <x:c r="B176" s="50" t="str">
+        <x:v>Chromium CI / serveur Vite HTTP</x:v>
+      </x:c>
+      <x:c r="C176" s="50" t="str">
+        <x:v>20/20 réussis</x:v>
+      </x:c>
+      <x:c r="D176" s="50" t="str">
+        <x:v>14 nouveaux parcours + 6 régressions</x:v>
+      </x:c>
+      <x:c r="E176" s="50" t="str">
+        <x:v>10 protocoles, 4 approches Nexus et 6 sélections/cadrages FPS existants.</x:v>
+      </x:c>
+      <x:c r="F176" s="50" t="str">
+        <x:v>Comptes/cibles préparés, horloge virtuelle. Médias secondaires absents du checkout non certifiés.</x:v>
+      </x:c>
+      <x:c r="G176" s="50" t="str">
+        <x:v>https://github.com/darknigthmare/multiverse-breach/actions/runs/40719252474</x:v>
+      </x:c>
+      <x:c r="H176" s="50" t="str">
+        <x:v>scripts/browserExtinctionProtocols.py / scripts/browserExtinctionCatalog.py</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12686,7 +13049,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1c3b11876894089"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13c76147bf8a45e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>